<commit_message>
BOM review ho gaya ha jin parts LCSC Link Add ha wo highlight kr diye han
</commit_message>
<xml_diff>
--- a/BOM/Digikey_BOM.xlsx
+++ b/BOM/Digikey_BOM.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="284">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="283">
   <si>
     <t>Description</t>
   </si>
@@ -697,9 +697,6 @@
   </si>
   <si>
     <t>--------</t>
-  </si>
-  <si>
-    <t>ZRB18AR61E106ME01L</t>
   </si>
   <si>
     <t xml:space="preserve">Diodes </t>
@@ -1068,7 +1065,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="27">
+  <borders count="28">
     <border>
       <left/>
       <right/>
@@ -1274,19 +1271,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top/>
@@ -1395,6 +1379,32 @@
         <color indexed="64"/>
       </right>
       <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
         <color indexed="64"/>
       </top>
       <bottom/>
@@ -1405,7 +1415,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="145">
+  <cellXfs count="152">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1487,9 +1497,6 @@
     <xf numFmtId="0" fontId="11" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="166" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1520,30 +1527,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1577,7 +1560,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1593,19 +1575,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="24" xfId="1" quotePrefix="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="23" xfId="1" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1620,215 +1602,266 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="1" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="1" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="20" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="21" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="21" xfId="1" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="13" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="10" xfId="1" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="21" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="23" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="18" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="17" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="17" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="17" xfId="1" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="22" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="23" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="23" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="23" xfId="1" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="18" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="21" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="1" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="1" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="23" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="15" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="21" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="22" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="22" xfId="1" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="13" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="10" xfId="1" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="22" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="24" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="19" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="18" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="18" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="18" xfId="1" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="23" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="24" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="24" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="24" xfId="1" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="5" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2117,10 +2150,10 @@
   <cols>
     <col min="1" max="1" width="6.140625" style="19" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.42578125" customWidth="1"/>
-    <col min="3" max="3" width="40.85546875" style="32" customWidth="1"/>
+    <col min="3" max="3" width="40.85546875" style="31" customWidth="1"/>
     <col min="4" max="4" width="31.5703125" style="19" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.28515625" style="33" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="25.28515625" style="33" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.28515625" style="32" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="25.28515625" style="32" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="19.140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="18.7109375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="7.28515625" style="19" bestFit="1" customWidth="1"/>
@@ -2139,29 +2172,29 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="133" t="s">
         <v>77</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
-      <c r="H1" s="46"/>
-      <c r="I1" s="46"/>
-      <c r="J1" s="46"/>
-      <c r="K1" s="46"/>
-      <c r="L1" s="46"/>
-      <c r="M1" s="46"/>
-      <c r="N1" s="46"/>
-      <c r="O1" s="46"/>
-      <c r="P1" s="46"/>
-      <c r="Q1" s="46"/>
-      <c r="R1" s="46"/>
-      <c r="S1" s="46"/>
-      <c r="T1" s="46"/>
-      <c r="U1" s="47"/>
+      <c r="B1" s="134"/>
+      <c r="C1" s="134"/>
+      <c r="D1" s="134"/>
+      <c r="E1" s="134"/>
+      <c r="F1" s="134"/>
+      <c r="G1" s="134"/>
+      <c r="H1" s="134"/>
+      <c r="I1" s="134"/>
+      <c r="J1" s="134"/>
+      <c r="K1" s="134"/>
+      <c r="L1" s="134"/>
+      <c r="M1" s="134"/>
+      <c r="N1" s="134"/>
+      <c r="O1" s="134"/>
+      <c r="P1" s="134"/>
+      <c r="Q1" s="134"/>
+      <c r="R1" s="134"/>
+      <c r="S1" s="134"/>
+      <c r="T1" s="134"/>
+      <c r="U1" s="135"/>
     </row>
     <row r="2" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -2232,10 +2265,10 @@
       <c r="A3" s="28">
         <v>1</v>
       </c>
-      <c r="B3" s="41" t="s">
+      <c r="B3" s="136" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="60" t="s">
+      <c r="C3" s="50" t="s">
         <v>82</v>
       </c>
       <c r="D3" s="23" t="s">
@@ -2256,7 +2289,7 @@
       <c r="I3" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="J3" s="61">
+      <c r="J3" s="51">
         <v>22</v>
       </c>
       <c r="K3" s="4">
@@ -2271,7 +2304,7 @@
         <f>J3*1000</f>
         <v>22000</v>
       </c>
-      <c r="N3" s="35" t="s">
+      <c r="N3" s="34" t="s">
         <v>17</v>
       </c>
       <c r="O3" s="13">
@@ -2303,69 +2336,69 @@
       <c r="A4" s="28">
         <v>2</v>
       </c>
-      <c r="B4" s="42"/>
-      <c r="C4" s="78" t="s">
+      <c r="B4" s="137"/>
+      <c r="C4" s="67" t="s">
         <v>86</v>
       </c>
-      <c r="D4" s="79" t="s">
+      <c r="D4" s="68" t="s">
         <v>87</v>
       </c>
-      <c r="E4" s="79" t="s">
+      <c r="E4" s="68" t="s">
         <v>88</v>
       </c>
-      <c r="F4" s="79" t="s">
+      <c r="F4" s="68" t="s">
         <v>89</v>
       </c>
-      <c r="G4" s="80" t="s">
+      <c r="G4" s="69" t="s">
         <v>219</v>
       </c>
-      <c r="H4" s="81" t="s">
+      <c r="H4" s="70" t="s">
         <v>220</v>
       </c>
-      <c r="I4" s="79" t="s">
+      <c r="I4" s="68" t="s">
         <v>21</v>
       </c>
-      <c r="J4" s="82">
+      <c r="J4" s="71">
         <v>6</v>
       </c>
-      <c r="K4" s="49">
+      <c r="K4" s="40">
         <f t="shared" ref="K4:K51" si="0">J4*5</f>
         <v>30</v>
       </c>
-      <c r="L4" s="49">
+      <c r="L4" s="40">
         <f t="shared" ref="L4:L51" si="1">J4*100</f>
         <v>600</v>
       </c>
-      <c r="M4" s="49">
+      <c r="M4" s="40">
         <f t="shared" ref="M4:M51" si="2">J4*1000</f>
         <v>6000</v>
       </c>
-      <c r="N4" s="83" t="s">
-        <v>257</v>
-      </c>
-      <c r="O4" s="84">
+      <c r="N4" s="72" t="s">
+        <v>256</v>
+      </c>
+      <c r="O4" s="73">
         <v>0.26250000000000001</v>
       </c>
-      <c r="P4" s="84">
-        <f t="shared" ref="P4:P51" si="3">O4*J4</f>
-        <v>1.5750000000000002</v>
-      </c>
-      <c r="Q4" s="84">
+      <c r="P4" s="14">
+        <f t="shared" ref="P4:P51" si="3">O4*K4</f>
+        <v>7.875</v>
+      </c>
+      <c r="Q4" s="73">
         <v>0.18060000000000001</v>
       </c>
-      <c r="R4" s="84">
+      <c r="R4" s="73">
         <f t="shared" ref="R4:R51" si="4">Q4*L4</f>
         <v>108.36</v>
       </c>
-      <c r="S4" s="84">
+      <c r="S4" s="73">
         <v>0.15939999999999999</v>
       </c>
-      <c r="T4" s="84">
+      <c r="T4" s="73">
         <f t="shared" ref="T4:T51" si="5">S4*M4</f>
         <v>956.39999999999986</v>
       </c>
-      <c r="U4" s="94" t="s">
-        <v>276</v>
+      <c r="U4" s="82" t="s">
+        <v>275</v>
       </c>
       <c r="V4" s="3"/>
       <c r="W4" s="3"/>
@@ -2374,68 +2407,68 @@
       <c r="A5" s="28">
         <v>3</v>
       </c>
-      <c r="B5" s="42"/>
-      <c r="C5" s="78" t="s">
+      <c r="B5" s="137"/>
+      <c r="C5" s="67" t="s">
         <v>90</v>
       </c>
-      <c r="D5" s="79" t="s">
+      <c r="D5" s="68" t="s">
         <v>91</v>
       </c>
-      <c r="E5" s="79" t="s">
+      <c r="E5" s="68" t="s">
         <v>108</v>
       </c>
-      <c r="F5" s="79" t="s">
+      <c r="F5" s="68" t="s">
         <v>92</v>
       </c>
-      <c r="G5" s="80" t="s">
+      <c r="G5" s="69" t="s">
         <v>221</v>
       </c>
-      <c r="H5" s="81" t="s">
-        <v>222</v>
-      </c>
-      <c r="I5" s="79" t="s">
+      <c r="H5" s="70" t="s">
+        <v>222</v>
+      </c>
+      <c r="I5" s="68" t="s">
         <v>22</v>
       </c>
-      <c r="J5" s="82">
+      <c r="J5" s="71">
         <v>3</v>
       </c>
-      <c r="K5" s="49">
+      <c r="K5" s="40">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="L5" s="49">
+      <c r="L5" s="40">
         <f t="shared" si="1"/>
         <v>300</v>
       </c>
-      <c r="M5" s="49">
+      <c r="M5" s="40">
         <f t="shared" si="2"/>
         <v>3000</v>
       </c>
-      <c r="N5" s="83" t="s">
-        <v>257</v>
-      </c>
-      <c r="O5" s="84">
+      <c r="N5" s="72" t="s">
+        <v>256</v>
+      </c>
+      <c r="O5" s="73">
         <v>8.3000000000000004E-2</v>
       </c>
-      <c r="P5" s="84">
+      <c r="P5" s="14">
         <f t="shared" si="3"/>
-        <v>0.249</v>
-      </c>
-      <c r="Q5" s="84">
+        <v>1.2450000000000001</v>
+      </c>
+      <c r="Q5" s="73">
         <v>6.0900000000000003E-2</v>
       </c>
-      <c r="R5" s="84">
+      <c r="R5" s="73">
         <f t="shared" si="4"/>
         <v>18.27</v>
       </c>
-      <c r="S5" s="85">
+      <c r="S5" s="74">
         <v>4.7600000000000003E-2</v>
       </c>
-      <c r="T5" s="84">
+      <c r="T5" s="73">
         <f t="shared" si="5"/>
         <v>142.80000000000001</v>
       </c>
-      <c r="U5" s="37"/>
+      <c r="U5" s="36"/>
       <c r="V5" s="3"/>
       <c r="W5" s="3"/>
     </row>
@@ -2443,8 +2476,8 @@
       <c r="A6" s="28">
         <v>4</v>
       </c>
-      <c r="B6" s="42"/>
-      <c r="C6" s="56" t="s">
+      <c r="B6" s="137"/>
+      <c r="C6" s="47" t="s">
         <v>93</v>
       </c>
       <c r="D6" s="24" t="s">
@@ -2465,7 +2498,7 @@
       <c r="I6" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="J6" s="48">
+      <c r="J6" s="39">
         <v>1</v>
       </c>
       <c r="K6" s="7">
@@ -2488,7 +2521,7 @@
       </c>
       <c r="P6" s="14">
         <f t="shared" si="3"/>
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="Q6" s="14">
         <v>2.5999999999999999E-2</v>
@@ -2512,8 +2545,8 @@
       <c r="A7" s="28">
         <v>5</v>
       </c>
-      <c r="B7" s="42"/>
-      <c r="C7" s="56" t="s">
+      <c r="B7" s="137"/>
+      <c r="C7" s="47" t="s">
         <v>95</v>
       </c>
       <c r="D7" s="24" t="s">
@@ -2534,7 +2567,7 @@
       <c r="I7" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="J7" s="48">
+      <c r="J7" s="39">
         <v>2</v>
       </c>
       <c r="K7" s="7">
@@ -2557,7 +2590,7 @@
       </c>
       <c r="P7" s="14">
         <f t="shared" si="3"/>
-        <v>0.192</v>
+        <v>0.96</v>
       </c>
       <c r="Q7" s="14">
         <v>4.4999999999999998E-2</v>
@@ -2581,8 +2614,8 @@
       <c r="A8" s="28">
         <v>6</v>
       </c>
-      <c r="B8" s="42"/>
-      <c r="C8" s="56" t="s">
+      <c r="B8" s="137"/>
+      <c r="C8" s="47" t="s">
         <v>98</v>
       </c>
       <c r="D8" s="24" t="s">
@@ -2603,7 +2636,7 @@
       <c r="I8" s="24" t="s">
         <v>80</v>
       </c>
-      <c r="J8" s="48">
+      <c r="J8" s="39">
         <v>1</v>
       </c>
       <c r="K8" s="7">
@@ -2626,7 +2659,7 @@
       </c>
       <c r="P8" s="14">
         <f t="shared" si="3"/>
-        <v>0.17</v>
+        <v>0.85000000000000009</v>
       </c>
       <c r="Q8" s="14">
         <v>5.8000000000000003E-2</v>
@@ -2650,8 +2683,8 @@
       <c r="A9" s="28">
         <v>7</v>
       </c>
-      <c r="B9" s="42"/>
-      <c r="C9" s="56" t="s">
+      <c r="B9" s="137"/>
+      <c r="C9" s="47" t="s">
         <v>102</v>
       </c>
       <c r="D9" s="24" t="s">
@@ -2660,19 +2693,19 @@
       <c r="E9" s="24" t="s">
         <v>84</v>
       </c>
-      <c r="F9" s="57" t="s">
+      <c r="F9" s="24" t="s">
         <v>104</v>
       </c>
       <c r="G9" s="6" t="s">
         <v>213</v>
       </c>
       <c r="H9" s="21" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="I9" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="J9" s="48">
+      <c r="J9" s="39">
         <v>2</v>
       </c>
       <c r="K9" s="7">
@@ -2688,30 +2721,30 @@
         <v>2000</v>
       </c>
       <c r="N9" s="27" t="s">
-        <v>17</v>
+        <v>256</v>
       </c>
       <c r="O9" s="14">
-        <v>0.35599999999999998</v>
+        <v>8.8499999999999995E-2</v>
       </c>
       <c r="P9" s="14">
         <f t="shared" si="3"/>
-        <v>0.71199999999999997</v>
+        <v>0.88500000000000001</v>
       </c>
       <c r="Q9" s="14">
-        <v>0.23469999999999999</v>
+        <v>6.5699999999999995E-2</v>
       </c>
       <c r="R9" s="14">
         <f t="shared" si="4"/>
-        <v>46.94</v>
+        <v>13.139999999999999</v>
       </c>
       <c r="S9" s="14">
-        <v>0.14779999999999999</v>
+        <v>6.2199999999999998E-2</v>
       </c>
       <c r="T9" s="14">
         <f t="shared" si="5"/>
-        <v>295.59999999999997</v>
-      </c>
-      <c r="U9" s="70"/>
+        <v>124.39999999999999</v>
+      </c>
+      <c r="U9" s="60"/>
       <c r="V9" s="3"/>
       <c r="W9" s="3"/>
     </row>
@@ -2719,17 +2752,17 @@
       <c r="A10" s="28">
         <v>8</v>
       </c>
-      <c r="B10" s="43"/>
-      <c r="C10" s="62" t="s">
+      <c r="B10" s="138"/>
+      <c r="C10" s="52" t="s">
         <v>105</v>
       </c>
-      <c r="D10" s="63" t="s">
+      <c r="D10" s="53" t="s">
         <v>106</v>
       </c>
-      <c r="E10" s="63" t="s">
+      <c r="E10" s="53" t="s">
         <v>84</v>
       </c>
-      <c r="F10" s="63" t="s">
+      <c r="F10" s="53" t="s">
         <v>107</v>
       </c>
       <c r="G10" s="9" t="s">
@@ -2738,10 +2771,10 @@
       <c r="H10" s="22" t="s">
         <v>222</v>
       </c>
-      <c r="I10" s="63" t="s">
+      <c r="I10" s="53" t="s">
         <v>81</v>
       </c>
-      <c r="J10" s="64">
+      <c r="J10" s="54">
         <v>1</v>
       </c>
       <c r="K10" s="10">
@@ -2756,7 +2789,7 @@
         <f t="shared" si="2"/>
         <v>1000</v>
       </c>
-      <c r="N10" s="36" t="s">
+      <c r="N10" s="35" t="s">
         <v>17</v>
       </c>
       <c r="O10" s="15">
@@ -2764,7 +2797,7 @@
       </c>
       <c r="P10" s="15">
         <f t="shared" si="3"/>
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="Q10" s="15">
         <v>2.4199999999999999E-2</v>
@@ -2788,31 +2821,31 @@
       <c r="A11" s="28">
         <v>9</v>
       </c>
-      <c r="B11" s="41" t="s">
+      <c r="B11" s="137" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="95" t="s">
-        <v>259</v>
-      </c>
-      <c r="D11" s="86" t="s">
+      <c r="C11" s="144" t="s">
+        <v>258</v>
+      </c>
+      <c r="D11" s="87" t="s">
         <v>109</v>
       </c>
-      <c r="E11" s="86" t="s">
+      <c r="E11" s="87" t="s">
         <v>23</v>
       </c>
-      <c r="F11" s="86" t="s">
+      <c r="F11" s="87" t="s">
         <v>45</v>
       </c>
-      <c r="G11" s="87" t="s">
-        <v>258</v>
-      </c>
-      <c r="H11" s="81" t="s">
-        <v>222</v>
-      </c>
-      <c r="I11" s="81" t="s">
-        <v>222</v>
-      </c>
-      <c r="J11" s="88">
+      <c r="G11" s="103" t="s">
+        <v>257</v>
+      </c>
+      <c r="H11" s="145" t="s">
+        <v>222</v>
+      </c>
+      <c r="I11" s="145" t="s">
+        <v>222</v>
+      </c>
+      <c r="J11" s="146">
         <v>1</v>
       </c>
       <c r="K11" s="89">
@@ -2828,14 +2861,14 @@
         <v>1000</v>
       </c>
       <c r="N11" s="90" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="O11" s="91">
         <v>7.5499999999999998E-2</v>
       </c>
-      <c r="P11" s="91">
+      <c r="P11" s="142">
         <f t="shared" si="3"/>
-        <v>7.5499999999999998E-2</v>
+        <v>0.3775</v>
       </c>
       <c r="Q11" s="91">
         <v>5.79E-2</v>
@@ -2851,7 +2884,7 @@
         <f t="shared" si="5"/>
         <v>45.3</v>
       </c>
-      <c r="U11" s="92"/>
+      <c r="U11" s="106"/>
       <c r="V11" s="3"/>
       <c r="W11" s="3"/>
     </row>
@@ -2859,69 +2892,69 @@
       <c r="A12" s="28">
         <v>10</v>
       </c>
-      <c r="B12" s="42"/>
-      <c r="C12" s="78" t="s">
+      <c r="B12" s="137"/>
+      <c r="C12" s="67" t="s">
         <v>110</v>
       </c>
-      <c r="D12" s="79" t="s">
+      <c r="D12" s="68" t="s">
         <v>111</v>
       </c>
-      <c r="E12" s="81" t="s">
+      <c r="E12" s="70" t="s">
+        <v>259</v>
+      </c>
+      <c r="F12" s="68" t="s">
+        <v>112</v>
+      </c>
+      <c r="G12" s="81" t="s">
         <v>260</v>
       </c>
-      <c r="F12" s="79" t="s">
-        <v>112</v>
-      </c>
-      <c r="G12" s="93" t="s">
-        <v>261</v>
-      </c>
-      <c r="H12" s="81" t="s">
-        <v>222</v>
-      </c>
-      <c r="I12" s="81" t="s">
-        <v>222</v>
-      </c>
-      <c r="J12" s="82">
+      <c r="H12" s="70" t="s">
+        <v>222</v>
+      </c>
+      <c r="I12" s="70" t="s">
+        <v>222</v>
+      </c>
+      <c r="J12" s="71">
         <v>1</v>
       </c>
-      <c r="K12" s="49">
+      <c r="K12" s="40">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L12" s="49">
+      <c r="L12" s="40">
         <f t="shared" si="1"/>
         <v>100</v>
       </c>
-      <c r="M12" s="49">
+      <c r="M12" s="40">
         <f t="shared" si="2"/>
         <v>1000</v>
       </c>
-      <c r="N12" s="83" t="s">
-        <v>257</v>
-      </c>
-      <c r="O12" s="84">
+      <c r="N12" s="72" t="s">
+        <v>256</v>
+      </c>
+      <c r="O12" s="73">
         <v>1.83E-2</v>
       </c>
-      <c r="P12" s="84">
+      <c r="P12" s="14">
         <f t="shared" si="3"/>
+        <v>9.1499999999999998E-2</v>
+      </c>
+      <c r="Q12" s="73">
         <v>1.83E-2</v>
       </c>
-      <c r="Q12" s="84">
-        <v>1.83E-2</v>
-      </c>
-      <c r="R12" s="84">
+      <c r="R12" s="73">
         <f t="shared" si="4"/>
         <v>1.83</v>
       </c>
-      <c r="S12" s="84">
+      <c r="S12" s="73">
         <v>1.23E-2</v>
       </c>
-      <c r="T12" s="84">
+      <c r="T12" s="73">
         <f t="shared" si="5"/>
         <v>12.3</v>
       </c>
-      <c r="U12" s="94" t="s">
-        <v>262</v>
+      <c r="U12" s="82" t="s">
+        <v>261</v>
       </c>
       <c r="V12" s="3"/>
       <c r="W12" s="3"/>
@@ -2930,68 +2963,68 @@
       <c r="A13" s="28">
         <v>11</v>
       </c>
-      <c r="B13" s="43"/>
-      <c r="C13" s="62" t="s">
+      <c r="B13" s="137"/>
+      <c r="C13" s="147" t="s">
         <v>113</v>
       </c>
-      <c r="D13" s="63" t="s">
+      <c r="D13" s="55" t="s">
         <v>114</v>
       </c>
-      <c r="E13" s="63" t="s">
-        <v>225</v>
-      </c>
-      <c r="F13" s="63" t="s">
+      <c r="E13" s="55" t="s">
+        <v>224</v>
+      </c>
+      <c r="F13" s="55" t="s">
         <v>115</v>
       </c>
-      <c r="G13" s="9" t="s">
-        <v>224</v>
-      </c>
-      <c r="H13" s="22" t="s">
-        <v>222</v>
-      </c>
-      <c r="I13" s="22" t="s">
-        <v>222</v>
-      </c>
-      <c r="J13" s="64">
+      <c r="G13" s="56" t="s">
+        <v>223</v>
+      </c>
+      <c r="H13" s="148" t="s">
+        <v>222</v>
+      </c>
+      <c r="I13" s="148" t="s">
+        <v>222</v>
+      </c>
+      <c r="J13" s="149">
         <v>2</v>
       </c>
-      <c r="K13" s="10">
+      <c r="K13" s="57">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="L13" s="10">
+      <c r="L13" s="57">
         <f t="shared" si="1"/>
         <v>200</v>
       </c>
-      <c r="M13" s="10">
+      <c r="M13" s="57">
         <f t="shared" si="2"/>
         <v>2000</v>
       </c>
-      <c r="N13" s="36" t="s">
+      <c r="N13" s="58" t="s">
         <v>17</v>
       </c>
-      <c r="O13" s="15">
+      <c r="O13" s="59">
         <v>0.35199999999999998</v>
       </c>
-      <c r="P13" s="15">
+      <c r="P13" s="59">
         <f t="shared" si="3"/>
-        <v>0.70399999999999996</v>
-      </c>
-      <c r="Q13" s="15">
+        <v>3.5199999999999996</v>
+      </c>
+      <c r="Q13" s="59">
         <v>0.1993</v>
       </c>
-      <c r="R13" s="15">
+      <c r="R13" s="59">
         <f t="shared" si="4"/>
         <v>39.86</v>
       </c>
-      <c r="S13" s="15">
+      <c r="S13" s="59">
         <v>0.1012</v>
       </c>
-      <c r="T13" s="15">
+      <c r="T13" s="59">
         <f t="shared" si="5"/>
         <v>202.4</v>
       </c>
-      <c r="U13" s="12"/>
+      <c r="U13" s="66"/>
       <c r="V13" s="3"/>
       <c r="W13" s="3"/>
     </row>
@@ -2999,82 +3032,82 @@
       <c r="A14" s="28">
         <v>12</v>
       </c>
-      <c r="B14" s="41" t="s">
+      <c r="B14" s="136" t="s">
         <v>30</v>
       </c>
-      <c r="C14" s="96" t="s">
+      <c r="C14" s="83" t="s">
         <v>116</v>
       </c>
-      <c r="D14" s="86" t="s">
+      <c r="D14" s="75" t="s">
         <v>28</v>
       </c>
-      <c r="E14" s="86" t="s">
+      <c r="E14" s="75" t="s">
         <v>117</v>
       </c>
-      <c r="F14" s="86" t="s">
+      <c r="F14" s="75" t="s">
         <v>49</v>
       </c>
-      <c r="G14" s="87" t="s">
-        <v>263</v>
-      </c>
-      <c r="H14" s="86" t="s">
-        <v>222</v>
-      </c>
-      <c r="I14" s="86" t="s">
+      <c r="G14" s="76" t="s">
+        <v>262</v>
+      </c>
+      <c r="H14" s="75" t="s">
+        <v>222</v>
+      </c>
+      <c r="I14" s="75" t="s">
         <v>31</v>
       </c>
-      <c r="J14" s="97">
+      <c r="J14" s="84">
         <v>1</v>
       </c>
-      <c r="K14" s="89">
+      <c r="K14" s="78">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L14" s="89">
+      <c r="L14" s="78">
         <f t="shared" si="1"/>
         <v>100</v>
       </c>
-      <c r="M14" s="89">
+      <c r="M14" s="78">
         <f t="shared" si="2"/>
         <v>1000</v>
       </c>
-      <c r="N14" s="90" t="s">
-        <v>257</v>
-      </c>
-      <c r="O14" s="91">
+      <c r="N14" s="79" t="s">
+        <v>256</v>
+      </c>
+      <c r="O14" s="80">
         <v>4.9000000000000002E-2</v>
       </c>
-      <c r="P14" s="91">
+      <c r="P14" s="13">
         <f t="shared" si="3"/>
-        <v>4.9000000000000002E-2</v>
-      </c>
-      <c r="Q14" s="91">
+        <v>0.245</v>
+      </c>
+      <c r="Q14" s="80">
         <v>3.9100000000000003E-2</v>
       </c>
-      <c r="R14" s="91">
+      <c r="R14" s="80">
         <f t="shared" si="4"/>
         <v>3.91</v>
       </c>
-      <c r="S14" s="91">
+      <c r="S14" s="80">
         <v>2.4899999999999999E-2</v>
       </c>
-      <c r="T14" s="91">
+      <c r="T14" s="80">
         <f t="shared" si="5"/>
         <v>24.9</v>
       </c>
-      <c r="U14" s="98" t="s">
-        <v>264</v>
+      <c r="U14" s="85" t="s">
+        <v>263</v>
       </c>
       <c r="V14" s="3"/>
       <c r="W14" s="3"/>
     </row>
-    <row r="15" spans="1:23" s="55" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:23" s="46" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="28">
         <v>13</v>
       </c>
-      <c r="B15" s="42"/>
-      <c r="C15" s="58" t="s">
-        <v>226</v>
+      <c r="B15" s="137"/>
+      <c r="C15" s="49" t="s">
+        <v>225</v>
       </c>
       <c r="D15" s="24" t="s">
         <v>29</v>
@@ -3094,7 +3127,7 @@
       <c r="I15" s="24" t="s">
         <v>47</v>
       </c>
-      <c r="J15" s="50">
+      <c r="J15" s="41">
         <v>1</v>
       </c>
       <c r="K15" s="7">
@@ -3105,62 +3138,62 @@
         <f t="shared" si="1"/>
         <v>100</v>
       </c>
-      <c r="M15" s="51">
+      <c r="M15" s="42">
         <f t="shared" si="2"/>
         <v>1000</v>
       </c>
-      <c r="N15" s="52" t="s">
+      <c r="N15" s="43" t="s">
         <v>17</v>
       </c>
-      <c r="O15" s="53">
+      <c r="O15" s="44">
         <v>0.48</v>
       </c>
       <c r="P15" s="14">
         <f t="shared" si="3"/>
-        <v>0.48</v>
-      </c>
-      <c r="Q15" s="53">
+        <v>2.4</v>
+      </c>
+      <c r="Q15" s="44">
         <v>0.29339999999999999</v>
       </c>
       <c r="R15" s="14">
         <f t="shared" si="4"/>
         <v>29.34</v>
       </c>
-      <c r="S15" s="53">
+      <c r="S15" s="44">
         <v>0.25074000000000002</v>
       </c>
       <c r="T15" s="14">
         <f t="shared" si="5"/>
         <v>250.74</v>
       </c>
-      <c r="U15" s="72"/>
-      <c r="V15" s="54"/>
-      <c r="W15" s="54"/>
+      <c r="U15" s="62"/>
+      <c r="V15" s="45"/>
+      <c r="W15" s="45"/>
     </row>
     <row r="16" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="28">
         <v>14</v>
       </c>
-      <c r="B16" s="43"/>
-      <c r="C16" s="73" t="s">
+      <c r="B16" s="138"/>
+      <c r="C16" s="63" t="s">
+        <v>226</v>
+      </c>
+      <c r="D16" s="53" t="s">
+        <v>46</v>
+      </c>
+      <c r="E16" s="53" t="s">
+        <v>108</v>
+      </c>
+      <c r="F16" s="53" t="s">
+        <v>119</v>
+      </c>
+      <c r="G16" s="9" t="s">
         <v>227</v>
       </c>
-      <c r="D16" s="63" t="s">
-        <v>46</v>
-      </c>
-      <c r="E16" s="63" t="s">
-        <v>108</v>
-      </c>
-      <c r="F16" s="63" t="s">
-        <v>119</v>
-      </c>
-      <c r="G16" s="9" t="s">
-        <v>228</v>
-      </c>
-      <c r="H16" s="63" t="s">
-        <v>222</v>
-      </c>
-      <c r="I16" s="63" t="s">
+      <c r="H16" s="53" t="s">
+        <v>222</v>
+      </c>
+      <c r="I16" s="53" t="s">
         <v>48</v>
       </c>
       <c r="J16" s="11">
@@ -3178,7 +3211,7 @@
         <f t="shared" si="2"/>
         <v>1000</v>
       </c>
-      <c r="N16" s="36" t="s">
+      <c r="N16" s="35" t="s">
         <v>17</v>
       </c>
       <c r="O16" s="15">
@@ -3186,7 +3219,7 @@
       </c>
       <c r="P16" s="15">
         <f t="shared" si="3"/>
-        <v>0.39</v>
+        <v>1.9500000000000002</v>
       </c>
       <c r="Q16" s="15">
         <v>0.23680000000000001</v>
@@ -3210,70 +3243,70 @@
       <c r="A17" s="28">
         <v>15</v>
       </c>
-      <c r="B17" s="42" t="s">
+      <c r="B17" s="137" t="s">
         <v>73</v>
       </c>
-      <c r="C17" s="99" t="s">
+      <c r="C17" s="86" t="s">
         <v>120</v>
       </c>
-      <c r="D17" s="100" t="s">
+      <c r="D17" s="87" t="s">
         <v>121</v>
       </c>
-      <c r="E17" s="100" t="s">
+      <c r="E17" s="87" t="s">
         <v>122</v>
       </c>
-      <c r="F17" s="100" t="s">
+      <c r="F17" s="87" t="s">
         <v>123</v>
       </c>
-      <c r="G17" s="100" t="s">
-        <v>265</v>
-      </c>
-      <c r="H17" s="79" t="s">
-        <v>222</v>
-      </c>
-      <c r="I17" s="79" t="s">
-        <v>222</v>
-      </c>
-      <c r="J17" s="101">
+      <c r="G17" s="87" t="s">
+        <v>264</v>
+      </c>
+      <c r="H17" s="87" t="s">
+        <v>222</v>
+      </c>
+      <c r="I17" s="87" t="s">
+        <v>222</v>
+      </c>
+      <c r="J17" s="88">
         <v>4</v>
       </c>
-      <c r="K17" s="102">
+      <c r="K17" s="89">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="L17" s="102">
+      <c r="L17" s="89">
         <f t="shared" si="1"/>
         <v>400</v>
       </c>
-      <c r="M17" s="102">
+      <c r="M17" s="89">
         <f t="shared" si="2"/>
         <v>4000</v>
       </c>
-      <c r="N17" s="103" t="s">
-        <v>257</v>
-      </c>
-      <c r="O17" s="104">
+      <c r="N17" s="90" t="s">
+        <v>256</v>
+      </c>
+      <c r="O17" s="91">
         <v>1.52E-2</v>
       </c>
-      <c r="P17" s="104">
+      <c r="P17" s="142">
         <f t="shared" si="3"/>
-        <v>6.08E-2</v>
-      </c>
-      <c r="Q17" s="104">
+        <v>0.30399999999999999</v>
+      </c>
+      <c r="Q17" s="91">
         <v>1.52E-2</v>
       </c>
-      <c r="R17" s="104">
+      <c r="R17" s="91">
         <f t="shared" si="4"/>
         <v>6.08</v>
       </c>
-      <c r="S17" s="104">
+      <c r="S17" s="91">
         <v>1.0999999999999999E-2</v>
       </c>
-      <c r="T17" s="104">
+      <c r="T17" s="91">
         <f t="shared" si="5"/>
         <v>44</v>
       </c>
-      <c r="U17" s="105"/>
+      <c r="U17" s="92"/>
       <c r="V17" s="3"/>
       <c r="W17" s="3"/>
     </row>
@@ -3281,69 +3314,69 @@
       <c r="A18" s="28">
         <v>16</v>
       </c>
-      <c r="B18" s="42"/>
-      <c r="C18" s="138" t="s">
+      <c r="B18" s="137"/>
+      <c r="C18" s="125" t="s">
         <v>124</v>
       </c>
-      <c r="D18" s="117" t="s">
+      <c r="D18" s="104" t="s">
         <v>125</v>
       </c>
-      <c r="E18" s="117" t="s">
+      <c r="E18" s="104" t="s">
         <v>126</v>
       </c>
-      <c r="F18" s="117" t="s">
+      <c r="F18" s="104" t="s">
         <v>127</v>
       </c>
-      <c r="G18" s="117" t="s">
+      <c r="G18" s="104" t="s">
+        <v>276</v>
+      </c>
+      <c r="H18" s="126" t="s">
+        <v>222</v>
+      </c>
+      <c r="I18" s="127" t="s">
         <v>277</v>
       </c>
-      <c r="H18" s="139" t="s">
-        <v>222</v>
-      </c>
-      <c r="I18" s="140" t="s">
-        <v>278</v>
-      </c>
-      <c r="J18" s="141">
+      <c r="J18" s="128">
         <v>4</v>
       </c>
-      <c r="K18" s="142">
+      <c r="K18" s="129">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="L18" s="142">
+      <c r="L18" s="129">
         <f t="shared" si="1"/>
         <v>400</v>
       </c>
-      <c r="M18" s="142">
+      <c r="M18" s="129">
         <f t="shared" si="2"/>
         <v>4000</v>
       </c>
-      <c r="N18" s="143" t="s">
-        <v>257</v>
-      </c>
-      <c r="O18" s="144">
+      <c r="N18" s="130" t="s">
+        <v>256</v>
+      </c>
+      <c r="O18" s="131">
         <v>8.6E-3</v>
       </c>
-      <c r="P18" s="144">
+      <c r="P18" s="59">
         <f t="shared" si="3"/>
-        <v>3.44E-2</v>
-      </c>
-      <c r="Q18" s="144">
+        <v>0.17199999999999999</v>
+      </c>
+      <c r="Q18" s="131">
         <v>8.6E-3</v>
       </c>
-      <c r="R18" s="144">
+      <c r="R18" s="131">
         <f t="shared" si="4"/>
         <v>3.44</v>
       </c>
-      <c r="S18" s="144">
+      <c r="S18" s="131">
         <v>5.8999999999999999E-3</v>
       </c>
-      <c r="T18" s="144">
+      <c r="T18" s="131">
         <f t="shared" si="5"/>
         <v>23.599999999999998</v>
       </c>
-      <c r="U18" s="98" t="s">
-        <v>279</v>
+      <c r="U18" s="151" t="s">
+        <v>278</v>
       </c>
       <c r="V18" s="3"/>
       <c r="W18" s="3"/>
@@ -3352,17 +3385,17 @@
       <c r="A19" s="28">
         <v>17</v>
       </c>
-      <c r="B19" s="41" t="s">
+      <c r="B19" s="136" t="s">
         <v>27</v>
       </c>
-      <c r="C19" s="60" t="s">
+      <c r="C19" s="50" t="s">
         <v>128</v>
       </c>
       <c r="D19" s="23" t="s">
         <v>129</v>
       </c>
       <c r="E19" s="20" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F19" s="23" t="s">
         <v>50</v>
@@ -3376,7 +3409,7 @@
       <c r="I19" s="23" t="s">
         <v>222</v>
       </c>
-      <c r="J19" s="61">
+      <c r="J19" s="51">
         <v>1</v>
       </c>
       <c r="K19" s="4">
@@ -3391,7 +3424,7 @@
         <f t="shared" si="2"/>
         <v>1000</v>
       </c>
-      <c r="N19" s="35" t="s">
+      <c r="N19" s="34" t="s">
         <v>17</v>
       </c>
       <c r="O19" s="13">
@@ -3399,7 +3432,7 @@
       </c>
       <c r="P19" s="13">
         <f t="shared" si="3"/>
-        <v>0.5</v>
+        <v>2.5</v>
       </c>
       <c r="Q19" s="13">
         <v>0.27460000000000001</v>
@@ -3423,69 +3456,69 @@
       <c r="A20" s="28">
         <v>18</v>
       </c>
-      <c r="B20" s="42"/>
-      <c r="C20" s="78" t="s">
+      <c r="B20" s="137"/>
+      <c r="C20" s="67" t="s">
         <v>130</v>
       </c>
-      <c r="D20" s="79" t="s">
+      <c r="D20" s="68" t="s">
         <v>131</v>
       </c>
-      <c r="E20" s="79" t="s">
+      <c r="E20" s="68" t="s">
         <v>61</v>
       </c>
-      <c r="F20" s="79" t="s">
+      <c r="F20" s="68" t="s">
         <v>62</v>
       </c>
-      <c r="G20" s="80" t="s">
-        <v>266</v>
-      </c>
-      <c r="H20" s="86" t="s">
-        <v>222</v>
-      </c>
-      <c r="I20" s="86" t="s">
-        <v>222</v>
-      </c>
-      <c r="J20" s="82">
+      <c r="G20" s="69" t="s">
+        <v>265</v>
+      </c>
+      <c r="H20" s="75" t="s">
+        <v>222</v>
+      </c>
+      <c r="I20" s="75" t="s">
+        <v>222</v>
+      </c>
+      <c r="J20" s="71">
         <v>2</v>
       </c>
-      <c r="K20" s="49">
+      <c r="K20" s="40">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="L20" s="49">
+      <c r="L20" s="40">
         <f t="shared" si="1"/>
         <v>200</v>
       </c>
-      <c r="M20" s="49">
+      <c r="M20" s="40">
         <f t="shared" si="2"/>
         <v>2000</v>
       </c>
-      <c r="N20" s="83" t="s">
-        <v>257</v>
-      </c>
-      <c r="O20" s="84">
+      <c r="N20" s="72" t="s">
+        <v>256</v>
+      </c>
+      <c r="O20" s="73">
         <v>6.1499999999999999E-2</v>
       </c>
-      <c r="P20" s="84">
+      <c r="P20" s="14">
         <f t="shared" si="3"/>
-        <v>0.123</v>
-      </c>
-      <c r="Q20" s="106">
+        <v>0.61499999999999999</v>
+      </c>
+      <c r="Q20" s="93">
         <v>4.53E-2</v>
       </c>
-      <c r="R20" s="84">
+      <c r="R20" s="73">
         <f t="shared" si="4"/>
         <v>9.06</v>
       </c>
-      <c r="S20" s="84">
+      <c r="S20" s="73">
         <v>3.7499999999999999E-2</v>
       </c>
-      <c r="T20" s="84">
+      <c r="T20" s="73">
         <f t="shared" si="5"/>
         <v>75</v>
       </c>
-      <c r="U20" s="107" t="s">
-        <v>264</v>
+      <c r="U20" s="94" t="s">
+        <v>263</v>
       </c>
       <c r="V20" s="3"/>
       <c r="W20" s="3"/>
@@ -3494,69 +3527,69 @@
       <c r="A21" s="28">
         <v>19</v>
       </c>
-      <c r="B21" s="43"/>
-      <c r="C21" s="108" t="s">
+      <c r="B21" s="138"/>
+      <c r="C21" s="95" t="s">
         <v>132</v>
       </c>
-      <c r="D21" s="109" t="s">
+      <c r="D21" s="96" t="s">
         <v>133</v>
       </c>
-      <c r="E21" s="110" t="s">
-        <v>230</v>
-      </c>
-      <c r="F21" s="109" t="s">
+      <c r="E21" s="97" t="s">
+        <v>229</v>
+      </c>
+      <c r="F21" s="96" t="s">
         <v>134</v>
       </c>
-      <c r="G21" s="111" t="s">
-        <v>224</v>
-      </c>
-      <c r="H21" s="109" t="s">
-        <v>222</v>
-      </c>
-      <c r="I21" s="109" t="s">
-        <v>222</v>
-      </c>
-      <c r="J21" s="112">
+      <c r="G21" s="98" t="s">
+        <v>223</v>
+      </c>
+      <c r="H21" s="96" t="s">
+        <v>222</v>
+      </c>
+      <c r="I21" s="96" t="s">
+        <v>222</v>
+      </c>
+      <c r="J21" s="99">
         <v>1</v>
       </c>
-      <c r="K21" s="113">
+      <c r="K21" s="100">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L21" s="113">
+      <c r="L21" s="100">
         <f t="shared" si="1"/>
         <v>100</v>
       </c>
-      <c r="M21" s="113">
+      <c r="M21" s="100">
         <f t="shared" si="2"/>
         <v>1000</v>
       </c>
-      <c r="N21" s="114" t="s">
-        <v>257</v>
-      </c>
-      <c r="O21" s="115">
+      <c r="N21" s="101" t="s">
+        <v>256</v>
+      </c>
+      <c r="O21" s="102">
         <v>0.1489</v>
       </c>
-      <c r="P21" s="115">
+      <c r="P21" s="15">
         <f t="shared" si="3"/>
-        <v>0.1489</v>
-      </c>
-      <c r="Q21" s="115">
+        <v>0.74450000000000005</v>
+      </c>
+      <c r="Q21" s="102">
         <v>0.11360000000000001</v>
       </c>
-      <c r="R21" s="115">
+      <c r="R21" s="102">
         <f t="shared" si="4"/>
         <v>11.360000000000001</v>
       </c>
-      <c r="S21" s="115">
+      <c r="S21" s="102">
         <v>8.0600000000000005E-2</v>
       </c>
-      <c r="T21" s="115">
+      <c r="T21" s="102">
         <f t="shared" si="5"/>
         <v>80.600000000000009</v>
       </c>
-      <c r="U21" s="134" t="s">
-        <v>268</v>
+      <c r="U21" s="121" t="s">
+        <v>267</v>
       </c>
       <c r="V21" s="3"/>
       <c r="W21" s="3"/>
@@ -3565,10 +3598,10 @@
       <c r="A22" s="28">
         <v>20</v>
       </c>
-      <c r="B22" s="41" t="s">
+      <c r="B22" s="136" t="s">
         <v>16</v>
       </c>
-      <c r="C22" s="60" t="s">
+      <c r="C22" s="50" t="s">
         <v>135</v>
       </c>
       <c r="D22" s="23" t="s">
@@ -3589,7 +3622,7 @@
       <c r="I22" s="23" t="s">
         <v>54</v>
       </c>
-      <c r="J22" s="61">
+      <c r="J22" s="51">
         <v>5</v>
       </c>
       <c r="K22" s="4">
@@ -3604,7 +3637,7 @@
         <f t="shared" si="2"/>
         <v>5000</v>
       </c>
-      <c r="N22" s="35" t="s">
+      <c r="N22" s="34" t="s">
         <v>17</v>
       </c>
       <c r="O22" s="13">
@@ -3612,7 +3645,7 @@
       </c>
       <c r="P22" s="13">
         <f t="shared" si="3"/>
-        <v>0.12</v>
+        <v>0.6</v>
       </c>
       <c r="Q22" s="13">
         <v>9.7000000000000003E-3</v>
@@ -3636,8 +3669,8 @@
       <c r="A23" s="28">
         <v>21</v>
       </c>
-      <c r="B23" s="42"/>
-      <c r="C23" s="56" t="s">
+      <c r="B23" s="137"/>
+      <c r="C23" s="47" t="s">
         <v>139</v>
       </c>
       <c r="D23" s="24" t="s">
@@ -3658,7 +3691,7 @@
       <c r="I23" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="J23" s="48">
+      <c r="J23" s="39">
         <v>6</v>
       </c>
       <c r="K23" s="7">
@@ -3681,7 +3714,7 @@
       </c>
       <c r="P23" s="14">
         <f t="shared" si="3"/>
-        <v>0.14400000000000002</v>
+        <v>0.72</v>
       </c>
       <c r="Q23" s="14">
         <v>9.7000000000000003E-3</v>
@@ -3705,8 +3738,8 @@
       <c r="A24" s="28">
         <v>22</v>
       </c>
-      <c r="B24" s="42"/>
-      <c r="C24" s="56" t="s">
+      <c r="B24" s="137"/>
+      <c r="C24" s="47" t="s">
         <v>142</v>
       </c>
       <c r="D24" s="24" t="s">
@@ -3719,7 +3752,7 @@
         <v>143</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H24" s="24" t="s">
         <v>222</v>
@@ -3727,7 +3760,7 @@
       <c r="I24" s="24" t="s">
         <v>170</v>
       </c>
-      <c r="J24" s="48">
+      <c r="J24" s="39">
         <v>1</v>
       </c>
       <c r="K24" s="7">
@@ -3750,7 +3783,7 @@
       </c>
       <c r="P24" s="14">
         <f t="shared" si="3"/>
-        <v>1.03</v>
+        <v>5.15</v>
       </c>
       <c r="Q24" s="14">
         <v>0.66149999999999998</v>
@@ -3774,69 +3807,69 @@
       <c r="A25" s="28">
         <v>23</v>
       </c>
-      <c r="B25" s="42"/>
-      <c r="C25" s="78" t="s">
+      <c r="B25" s="137"/>
+      <c r="C25" s="67" t="s">
         <v>144</v>
       </c>
-      <c r="D25" s="79" t="s">
+      <c r="D25" s="68" t="s">
         <v>51</v>
       </c>
-      <c r="E25" s="79" t="s">
+      <c r="E25" s="68" t="s">
         <v>137</v>
       </c>
-      <c r="F25" s="79" t="s">
+      <c r="F25" s="68" t="s">
         <v>145</v>
       </c>
-      <c r="G25" s="80" t="s">
+      <c r="G25" s="69" t="s">
         <v>66</v>
       </c>
-      <c r="H25" s="79" t="s">
-        <v>222</v>
-      </c>
-      <c r="I25" s="79" t="s">
+      <c r="H25" s="68" t="s">
+        <v>222</v>
+      </c>
+      <c r="I25" s="68" t="s">
         <v>171</v>
       </c>
-      <c r="J25" s="82">
+      <c r="J25" s="71">
         <v>1</v>
       </c>
-      <c r="K25" s="49">
+      <c r="K25" s="40">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L25" s="49">
+      <c r="L25" s="40">
         <f t="shared" si="1"/>
         <v>100</v>
       </c>
-      <c r="M25" s="49">
+      <c r="M25" s="40">
         <f t="shared" si="2"/>
         <v>1000</v>
       </c>
-      <c r="N25" s="83" t="s">
-        <v>257</v>
-      </c>
-      <c r="O25" s="84">
+      <c r="N25" s="72" t="s">
+        <v>256</v>
+      </c>
+      <c r="O25" s="73">
         <v>1.2999999999999999E-3</v>
       </c>
-      <c r="P25" s="84">
+      <c r="P25" s="14">
         <f t="shared" si="3"/>
+        <v>6.4999999999999997E-3</v>
+      </c>
+      <c r="Q25" s="73">
         <v>1.2999999999999999E-3</v>
       </c>
-      <c r="Q25" s="84">
-        <v>1.2999999999999999E-3</v>
-      </c>
-      <c r="R25" s="84">
+      <c r="R25" s="73">
         <f t="shared" si="4"/>
         <v>0.13</v>
       </c>
-      <c r="S25" s="84">
+      <c r="S25" s="73">
         <v>8.9999999999999998E-4</v>
       </c>
-      <c r="T25" s="84">
+      <c r="T25" s="73">
         <f t="shared" si="5"/>
         <v>0.9</v>
       </c>
-      <c r="U25" s="94" t="s">
-        <v>267</v>
+      <c r="U25" s="82" t="s">
+        <v>266</v>
       </c>
       <c r="V25" s="3"/>
       <c r="W25" s="3"/>
@@ -3845,8 +3878,8 @@
       <c r="A26" s="28">
         <v>24</v>
       </c>
-      <c r="B26" s="42"/>
-      <c r="C26" s="56" t="s">
+      <c r="B26" s="137"/>
+      <c r="C26" s="47" t="s">
         <v>146</v>
       </c>
       <c r="D26" s="24" t="s">
@@ -3867,7 +3900,7 @@
       <c r="I26" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="J26" s="48">
+      <c r="J26" s="39">
         <v>7</v>
       </c>
       <c r="K26" s="7">
@@ -3890,7 +3923,7 @@
       </c>
       <c r="P26" s="14">
         <f t="shared" si="3"/>
-        <v>0.16800000000000001</v>
+        <v>0.84</v>
       </c>
       <c r="Q26" s="14">
         <v>9.7000000000000003E-3</v>
@@ -3914,69 +3947,69 @@
       <c r="A27" s="28">
         <v>25</v>
       </c>
-      <c r="B27" s="42"/>
-      <c r="C27" s="78" t="s">
+      <c r="B27" s="137"/>
+      <c r="C27" s="67" t="s">
         <v>149</v>
       </c>
-      <c r="D27" s="79" t="s">
+      <c r="D27" s="68" t="s">
         <v>150</v>
       </c>
-      <c r="E27" s="79" t="s">
+      <c r="E27" s="68" t="s">
         <v>151</v>
       </c>
-      <c r="F27" s="79" t="s">
+      <c r="F27" s="68" t="s">
         <v>152</v>
       </c>
-      <c r="G27" s="80" t="s">
+      <c r="G27" s="69" t="s">
         <v>66</v>
       </c>
-      <c r="H27" s="79" t="s">
-        <v>222</v>
-      </c>
-      <c r="I27" s="79" t="s">
+      <c r="H27" s="68" t="s">
+        <v>222</v>
+      </c>
+      <c r="I27" s="68" t="s">
         <v>172</v>
       </c>
-      <c r="J27" s="82">
+      <c r="J27" s="71">
         <v>1</v>
       </c>
-      <c r="K27" s="49">
+      <c r="K27" s="40">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L27" s="49">
+      <c r="L27" s="40">
         <f t="shared" si="1"/>
         <v>100</v>
       </c>
-      <c r="M27" s="49">
+      <c r="M27" s="40">
         <f t="shared" si="2"/>
         <v>1000</v>
       </c>
-      <c r="N27" s="83" t="s">
-        <v>257</v>
-      </c>
-      <c r="O27" s="84">
+      <c r="N27" s="72" t="s">
+        <v>256</v>
+      </c>
+      <c r="O27" s="73">
         <v>0.1472</v>
       </c>
-      <c r="P27" s="84">
+      <c r="P27" s="14">
         <f t="shared" si="3"/>
-        <v>0.1472</v>
-      </c>
-      <c r="Q27" s="84">
+        <v>0.73599999999999999</v>
+      </c>
+      <c r="Q27" s="73">
         <v>0.11310000000000001</v>
       </c>
-      <c r="R27" s="84">
+      <c r="R27" s="73">
         <f t="shared" si="4"/>
         <v>11.31</v>
       </c>
-      <c r="S27" s="84">
+      <c r="S27" s="73">
         <v>8.2500000000000004E-2</v>
       </c>
-      <c r="T27" s="84">
+      <c r="T27" s="73">
         <f t="shared" si="5"/>
         <v>82.5</v>
       </c>
-      <c r="U27" s="94" t="s">
-        <v>268</v>
+      <c r="U27" s="82" t="s">
+        <v>267</v>
       </c>
       <c r="V27" s="3"/>
       <c r="W27" s="3"/>
@@ -3985,8 +4018,8 @@
       <c r="A28" s="28">
         <v>26</v>
       </c>
-      <c r="B28" s="42"/>
-      <c r="C28" s="56" t="s">
+      <c r="B28" s="137"/>
+      <c r="C28" s="47" t="s">
         <v>153</v>
       </c>
       <c r="D28" s="24" t="s">
@@ -3999,7 +4032,7 @@
         <v>154</v>
       </c>
       <c r="G28" s="6" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="H28" s="24" t="s">
         <v>222</v>
@@ -4007,7 +4040,7 @@
       <c r="I28" s="24" t="s">
         <v>56</v>
       </c>
-      <c r="J28" s="48">
+      <c r="J28" s="39">
         <v>1</v>
       </c>
       <c r="K28" s="7">
@@ -4023,14 +4056,14 @@
         <v>1000</v>
       </c>
       <c r="N28" s="27" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="O28" s="14">
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="P28" s="14">
         <f t="shared" si="3"/>
-        <v>7.0000000000000007E-2</v>
+        <v>0.35000000000000003</v>
       </c>
       <c r="Q28" s="14">
         <v>1.9E-2</v>
@@ -4054,9 +4087,9 @@
       <c r="A29" s="28">
         <v>27</v>
       </c>
-      <c r="B29" s="42"/>
-      <c r="C29" s="58" t="s">
-        <v>234</v>
+      <c r="B29" s="137"/>
+      <c r="C29" s="49" t="s">
+        <v>233</v>
       </c>
       <c r="D29" s="24" t="s">
         <v>52</v>
@@ -4076,7 +4109,7 @@
       <c r="I29" s="24" t="s">
         <v>55</v>
       </c>
-      <c r="J29" s="48">
+      <c r="J29" s="39">
         <v>1</v>
       </c>
       <c r="K29" s="7">
@@ -4099,7 +4132,7 @@
       </c>
       <c r="P29" s="14">
         <f t="shared" si="3"/>
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="Q29" s="14">
         <v>1.17E-2</v>
@@ -4123,8 +4156,8 @@
       <c r="A30" s="28">
         <v>28</v>
       </c>
-      <c r="B30" s="42"/>
-      <c r="C30" s="56" t="s">
+      <c r="B30" s="137"/>
+      <c r="C30" s="47" t="s">
         <v>156</v>
       </c>
       <c r="D30" s="24" t="s">
@@ -4145,7 +4178,7 @@
       <c r="I30" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="J30" s="48">
+      <c r="J30" s="39">
         <v>3</v>
       </c>
       <c r="K30" s="7">
@@ -4168,7 +4201,7 @@
       </c>
       <c r="P30" s="14">
         <f t="shared" si="3"/>
-        <v>7.2000000000000008E-2</v>
+        <v>0.36</v>
       </c>
       <c r="Q30" s="14">
         <v>9.7000000000000003E-3</v>
@@ -4192,8 +4225,8 @@
       <c r="A31" s="28">
         <v>29</v>
       </c>
-      <c r="B31" s="42"/>
-      <c r="C31" s="56" t="s">
+      <c r="B31" s="137"/>
+      <c r="C31" s="47" t="s">
         <v>159</v>
       </c>
       <c r="D31" s="24" t="s">
@@ -4214,7 +4247,7 @@
       <c r="I31" s="24" t="s">
         <v>173</v>
       </c>
-      <c r="J31" s="48">
+      <c r="J31" s="39">
         <v>1</v>
       </c>
       <c r="K31" s="7">
@@ -4237,7 +4270,7 @@
       </c>
       <c r="P31" s="14">
         <f t="shared" si="3"/>
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="Q31" s="14">
         <v>8.0000000000000002E-3</v>
@@ -4253,7 +4286,7 @@
         <f t="shared" si="5"/>
         <v>3.6</v>
       </c>
-      <c r="U31" s="70"/>
+      <c r="U31" s="60"/>
       <c r="V31" s="3"/>
       <c r="W31" s="3"/>
     </row>
@@ -4261,9 +4294,9 @@
       <c r="A32" s="28">
         <v>30</v>
       </c>
-      <c r="B32" s="42"/>
-      <c r="C32" s="58" t="s">
-        <v>235</v>
+      <c r="B32" s="137"/>
+      <c r="C32" s="49" t="s">
+        <v>234</v>
       </c>
       <c r="D32" s="24" t="s">
         <v>161</v>
@@ -4275,7 +4308,7 @@
         <v>162</v>
       </c>
       <c r="G32" s="6" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="H32" s="24" t="s">
         <v>222</v>
@@ -4283,7 +4316,7 @@
       <c r="I32" s="24" t="s">
         <v>174</v>
       </c>
-      <c r="J32" s="48">
+      <c r="J32" s="39">
         <v>1</v>
       </c>
       <c r="K32" s="7">
@@ -4306,7 +4339,7 @@
       </c>
       <c r="P32" s="14">
         <f t="shared" si="3"/>
-        <v>0.27</v>
+        <v>1.35</v>
       </c>
       <c r="Q32" s="14">
         <v>8.7999999999999995E-2</v>
@@ -4330,8 +4363,8 @@
       <c r="A33" s="28">
         <v>31</v>
       </c>
-      <c r="B33" s="42"/>
-      <c r="C33" s="56" t="s">
+      <c r="B33" s="137"/>
+      <c r="C33" s="47" t="s">
         <v>163</v>
       </c>
       <c r="D33" s="24" t="s">
@@ -4340,19 +4373,19 @@
       <c r="E33" s="24" t="s">
         <v>137</v>
       </c>
-      <c r="F33" s="57" t="s">
+      <c r="F33" s="48" t="s">
         <v>165</v>
       </c>
       <c r="G33" s="6" t="s">
         <v>66</v>
       </c>
       <c r="H33" s="6" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="I33" s="24" t="s">
         <v>175</v>
       </c>
-      <c r="J33" s="48">
+      <c r="J33" s="39">
         <v>1</v>
       </c>
       <c r="K33" s="7">
@@ -4375,7 +4408,7 @@
       </c>
       <c r="P33" s="14">
         <f t="shared" si="3"/>
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="Q33" s="14">
         <v>1.14E-2</v>
@@ -4391,7 +4424,7 @@
         <f t="shared" si="5"/>
         <v>5.12</v>
       </c>
-      <c r="U33" s="70"/>
+      <c r="U33" s="60"/>
       <c r="V33" s="3"/>
       <c r="W33" s="3"/>
     </row>
@@ -4399,29 +4432,29 @@
       <c r="A34" s="28">
         <v>32</v>
       </c>
-      <c r="B34" s="43"/>
-      <c r="C34" s="62" t="s">
+      <c r="B34" s="138"/>
+      <c r="C34" s="52" t="s">
         <v>166</v>
       </c>
-      <c r="D34" s="63" t="s">
+      <c r="D34" s="53" t="s">
         <v>167</v>
       </c>
-      <c r="E34" s="63" t="s">
+      <c r="E34" s="53" t="s">
         <v>168</v>
       </c>
-      <c r="F34" s="63" t="s">
+      <c r="F34" s="53" t="s">
         <v>169</v>
       </c>
       <c r="G34" s="9" t="s">
-        <v>232</v>
-      </c>
-      <c r="H34" s="63" t="s">
-        <v>222</v>
-      </c>
-      <c r="I34" s="63" t="s">
+        <v>231</v>
+      </c>
+      <c r="H34" s="53" t="s">
+        <v>222</v>
+      </c>
+      <c r="I34" s="53" t="s">
         <v>176</v>
       </c>
-      <c r="J34" s="64">
+      <c r="J34" s="54">
         <v>4</v>
       </c>
       <c r="K34" s="10">
@@ -4436,7 +4469,7 @@
         <f t="shared" si="2"/>
         <v>4000</v>
       </c>
-      <c r="N34" s="36" t="s">
+      <c r="N34" s="35" t="s">
         <v>17</v>
       </c>
       <c r="O34" s="15">
@@ -4444,7 +4477,7 @@
       </c>
       <c r="P34" s="15">
         <f t="shared" si="3"/>
-        <v>2.536</v>
+        <v>12.68</v>
       </c>
       <c r="Q34" s="15">
         <v>0.36940000000000001</v>
@@ -4460,7 +4493,7 @@
         <f t="shared" si="5"/>
         <v>800.08</v>
       </c>
-      <c r="U34" s="71"/>
+      <c r="U34" s="61"/>
       <c r="V34" s="3"/>
       <c r="W34" s="3"/>
     </row>
@@ -4468,70 +4501,70 @@
       <c r="A35" s="28">
         <v>33</v>
       </c>
-      <c r="B35" s="42" t="s">
+      <c r="B35" s="137" t="s">
         <v>74</v>
       </c>
-      <c r="C35" s="99" t="s">
+      <c r="C35" s="86" t="s">
         <v>177</v>
       </c>
-      <c r="D35" s="100" t="s">
+      <c r="D35" s="87" t="s">
         <v>178</v>
       </c>
-      <c r="E35" s="100" t="s">
+      <c r="E35" s="87" t="s">
         <v>108</v>
       </c>
-      <c r="F35" s="100" t="s">
+      <c r="F35" s="87" t="s">
         <v>179</v>
       </c>
-      <c r="G35" s="116" t="s">
-        <v>269</v>
-      </c>
-      <c r="H35" s="117" t="s">
-        <v>222</v>
-      </c>
-      <c r="I35" s="117" t="s">
-        <v>222</v>
-      </c>
-      <c r="J35" s="118">
+      <c r="G35" s="103" t="s">
+        <v>268</v>
+      </c>
+      <c r="H35" s="108" t="s">
+        <v>222</v>
+      </c>
+      <c r="I35" s="108" t="s">
+        <v>222</v>
+      </c>
+      <c r="J35" s="105">
         <v>1</v>
       </c>
-      <c r="K35" s="102">
+      <c r="K35" s="89">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L35" s="102">
+      <c r="L35" s="89">
         <f t="shared" si="1"/>
         <v>100</v>
       </c>
-      <c r="M35" s="102">
+      <c r="M35" s="89">
         <f t="shared" si="2"/>
         <v>1000</v>
       </c>
-      <c r="N35" s="103" t="s">
-        <v>257</v>
-      </c>
-      <c r="O35" s="104">
+      <c r="N35" s="90" t="s">
+        <v>256</v>
+      </c>
+      <c r="O35" s="91">
         <v>5.1799999999999999E-2</v>
       </c>
-      <c r="P35" s="104">
+      <c r="P35" s="142">
         <f t="shared" si="3"/>
-        <v>5.1799999999999999E-2</v>
-      </c>
-      <c r="Q35" s="104">
+        <v>0.25900000000000001</v>
+      </c>
+      <c r="Q35" s="91">
         <v>3.7400000000000003E-2</v>
       </c>
-      <c r="R35" s="104">
+      <c r="R35" s="91">
         <f t="shared" si="4"/>
         <v>3.74</v>
       </c>
-      <c r="S35" s="104">
+      <c r="S35" s="91">
         <v>1.29E-2</v>
       </c>
-      <c r="T35" s="104">
+      <c r="T35" s="91">
         <f t="shared" si="5"/>
         <v>12.9</v>
       </c>
-      <c r="U35" s="119"/>
+      <c r="U35" s="106"/>
       <c r="V35" s="3"/>
       <c r="W35" s="3"/>
     </row>
@@ -4539,68 +4572,68 @@
       <c r="A36" s="28">
         <v>34</v>
       </c>
-      <c r="B36" s="42"/>
-      <c r="C36" s="74" t="s">
+      <c r="B36" s="137"/>
+      <c r="C36" s="64" t="s">
+        <v>236</v>
+      </c>
+      <c r="D36" s="55" t="s">
+        <v>180</v>
+      </c>
+      <c r="E36" s="55" t="s">
+        <v>108</v>
+      </c>
+      <c r="F36" s="55" t="s">
+        <v>58</v>
+      </c>
+      <c r="G36" s="56" t="s">
         <v>237</v>
       </c>
-      <c r="D36" s="65" t="s">
-        <v>180</v>
-      </c>
-      <c r="E36" s="65" t="s">
-        <v>108</v>
-      </c>
-      <c r="F36" s="65" t="s">
-        <v>58</v>
-      </c>
-      <c r="G36" s="66" t="s">
-        <v>238</v>
-      </c>
-      <c r="H36" s="65" t="s">
-        <v>222</v>
-      </c>
-      <c r="I36" s="65" t="s">
-        <v>222</v>
-      </c>
-      <c r="J36" s="75">
+      <c r="H36" s="55" t="s">
+        <v>222</v>
+      </c>
+      <c r="I36" s="55" t="s">
+        <v>222</v>
+      </c>
+      <c r="J36" s="65">
         <v>1</v>
       </c>
-      <c r="K36" s="67">
+      <c r="K36" s="57">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L36" s="67">
+      <c r="L36" s="57">
         <f t="shared" si="1"/>
         <v>100</v>
       </c>
-      <c r="M36" s="67">
+      <c r="M36" s="57">
         <f t="shared" si="2"/>
         <v>1000</v>
       </c>
-      <c r="N36" s="68" t="s">
-        <v>239</v>
-      </c>
-      <c r="O36" s="69">
+      <c r="N36" s="58" t="s">
+        <v>238</v>
+      </c>
+      <c r="O36" s="59">
         <v>0.48799999999999999</v>
       </c>
-      <c r="P36" s="69">
+      <c r="P36" s="59">
         <f t="shared" si="3"/>
-        <v>0.48799999999999999</v>
-      </c>
-      <c r="Q36" s="69">
+        <v>2.44</v>
+      </c>
+      <c r="Q36" s="59">
         <v>0.36399999999999999</v>
       </c>
-      <c r="R36" s="69">
+      <c r="R36" s="59">
         <f t="shared" si="4"/>
         <v>36.4</v>
       </c>
-      <c r="S36" s="69">
+      <c r="S36" s="59">
         <v>0.33200000000000002</v>
       </c>
-      <c r="T36" s="69">
+      <c r="T36" s="59">
         <f t="shared" si="5"/>
         <v>332</v>
       </c>
-      <c r="U36" s="76"/>
+      <c r="U36" s="66"/>
       <c r="V36" s="3"/>
       <c r="W36" s="3"/>
     </row>
@@ -4608,71 +4641,71 @@
       <c r="A37" s="28">
         <v>35</v>
       </c>
-      <c r="B37" s="41" t="s">
+      <c r="B37" s="136" t="s">
         <v>75</v>
       </c>
-      <c r="C37" s="96" t="s">
+      <c r="C37" s="83" t="s">
         <v>181</v>
       </c>
-      <c r="D37" s="86" t="s">
+      <c r="D37" s="75" t="s">
         <v>32</v>
       </c>
-      <c r="E37" s="86" t="s">
+      <c r="E37" s="75" t="s">
         <v>182</v>
       </c>
-      <c r="F37" s="86" t="s">
+      <c r="F37" s="75" t="s">
         <v>64</v>
       </c>
-      <c r="G37" s="87" t="s">
-        <v>280</v>
-      </c>
-      <c r="H37" s="86" t="s">
-        <v>222</v>
-      </c>
-      <c r="I37" s="86" t="s">
-        <v>222</v>
-      </c>
-      <c r="J37" s="88">
+      <c r="G37" s="76" t="s">
+        <v>279</v>
+      </c>
+      <c r="H37" s="75" t="s">
+        <v>222</v>
+      </c>
+      <c r="I37" s="75" t="s">
+        <v>222</v>
+      </c>
+      <c r="J37" s="77">
         <v>1</v>
       </c>
-      <c r="K37" s="89">
+      <c r="K37" s="78">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L37" s="89">
+      <c r="L37" s="78">
         <f t="shared" si="1"/>
         <v>100</v>
       </c>
-      <c r="M37" s="89">
+      <c r="M37" s="78">
         <f t="shared" si="2"/>
         <v>1000</v>
       </c>
-      <c r="N37" s="90" t="s">
-        <v>257</v>
-      </c>
-      <c r="O37" s="91">
+      <c r="N37" s="79" t="s">
+        <v>256</v>
+      </c>
+      <c r="O37" s="80">
         <v>4.8707000000000003</v>
       </c>
-      <c r="P37" s="91">
+      <c r="P37" s="13">
         <f t="shared" si="3"/>
-        <v>4.8707000000000003</v>
-      </c>
-      <c r="Q37" s="91">
+        <v>24.3535</v>
+      </c>
+      <c r="Q37" s="80">
         <v>3.2027000000000001</v>
       </c>
-      <c r="R37" s="91">
+      <c r="R37" s="80">
         <f t="shared" si="4"/>
         <v>320.27</v>
       </c>
-      <c r="S37" s="91">
+      <c r="S37" s="80">
         <v>3.0169000000000001</v>
       </c>
-      <c r="T37" s="91">
+      <c r="T37" s="80">
         <f t="shared" si="5"/>
         <v>3016.9</v>
       </c>
-      <c r="U37" s="132" t="s">
-        <v>281</v>
+      <c r="U37" s="119" t="s">
+        <v>280</v>
       </c>
       <c r="V37" s="3"/>
       <c r="W37" s="3"/>
@@ -4681,68 +4714,68 @@
       <c r="A38" s="28">
         <v>36</v>
       </c>
-      <c r="B38" s="42"/>
-      <c r="C38" s="78" t="s">
+      <c r="B38" s="137"/>
+      <c r="C38" s="67" t="s">
         <v>183</v>
       </c>
-      <c r="D38" s="79" t="s">
+      <c r="D38" s="68" t="s">
         <v>33</v>
       </c>
-      <c r="E38" s="79" t="s">
+      <c r="E38" s="68" t="s">
         <v>184</v>
       </c>
-      <c r="F38" s="79" t="s">
+      <c r="F38" s="68" t="s">
         <v>185</v>
       </c>
-      <c r="G38" s="80" t="s">
-        <v>270</v>
-      </c>
-      <c r="H38" s="79" t="s">
-        <v>222</v>
-      </c>
-      <c r="I38" s="79" t="s">
-        <v>222</v>
-      </c>
-      <c r="J38" s="82">
+      <c r="G38" s="69" t="s">
+        <v>269</v>
+      </c>
+      <c r="H38" s="68" t="s">
+        <v>222</v>
+      </c>
+      <c r="I38" s="68" t="s">
+        <v>222</v>
+      </c>
+      <c r="J38" s="71">
         <v>1</v>
       </c>
-      <c r="K38" s="49">
+      <c r="K38" s="40">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L38" s="49">
+      <c r="L38" s="40">
         <f t="shared" si="1"/>
         <v>100</v>
       </c>
-      <c r="M38" s="49">
+      <c r="M38" s="40">
         <f t="shared" si="2"/>
         <v>1000</v>
       </c>
-      <c r="N38" s="83" t="s">
-        <v>257</v>
-      </c>
-      <c r="O38" s="84">
+      <c r="N38" s="72" t="s">
+        <v>256</v>
+      </c>
+      <c r="O38" s="73">
         <v>0.37019999999999997</v>
       </c>
-      <c r="P38" s="84">
+      <c r="P38" s="14">
         <f t="shared" si="3"/>
-        <v>0.37019999999999997</v>
-      </c>
-      <c r="Q38" s="84">
+        <v>1.851</v>
+      </c>
+      <c r="Q38" s="73">
         <v>0.25190000000000001</v>
       </c>
-      <c r="R38" s="84">
+      <c r="R38" s="73">
         <f t="shared" si="4"/>
         <v>25.19</v>
       </c>
-      <c r="S38" s="84">
+      <c r="S38" s="73">
         <v>0.24160000000000001</v>
       </c>
-      <c r="T38" s="84">
+      <c r="T38" s="73">
         <f t="shared" si="5"/>
         <v>241.60000000000002</v>
       </c>
-      <c r="U38" s="37"/>
+      <c r="U38" s="36"/>
       <c r="V38" s="3"/>
       <c r="W38" s="3"/>
     </row>
@@ -4750,21 +4783,21 @@
       <c r="A39" s="28">
         <v>37</v>
       </c>
-      <c r="B39" s="42"/>
-      <c r="C39" s="58" t="s">
-        <v>241</v>
+      <c r="B39" s="137"/>
+      <c r="C39" s="49" t="s">
+        <v>240</v>
       </c>
       <c r="D39" s="24" t="s">
         <v>34</v>
       </c>
       <c r="E39" s="21" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="F39" s="24" t="s">
         <v>186</v>
       </c>
       <c r="G39" s="6" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="H39" s="24" t="s">
         <v>222</v>
@@ -4772,7 +4805,7 @@
       <c r="I39" s="24" t="s">
         <v>222</v>
       </c>
-      <c r="J39" s="48">
+      <c r="J39" s="39">
         <v>1</v>
       </c>
       <c r="K39" s="7">
@@ -4795,7 +4828,7 @@
       </c>
       <c r="P39" s="14">
         <f t="shared" si="3"/>
-        <v>0.48</v>
+        <v>2.4</v>
       </c>
       <c r="Q39" s="14">
         <v>0.2656</v>
@@ -4819,21 +4852,21 @@
       <c r="A40" s="28">
         <v>38</v>
       </c>
-      <c r="B40" s="42"/>
-      <c r="C40" s="56" t="s">
+      <c r="B40" s="137"/>
+      <c r="C40" s="47" t="s">
         <v>187</v>
       </c>
       <c r="D40" s="24" t="s">
         <v>35</v>
       </c>
       <c r="E40" s="21" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="F40" s="24" t="s">
         <v>188</v>
       </c>
       <c r="G40" s="6" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="H40" s="24" t="s">
         <v>222</v>
@@ -4841,7 +4874,7 @@
       <c r="I40" s="24" t="s">
         <v>222</v>
       </c>
-      <c r="J40" s="48">
+      <c r="J40" s="39">
         <v>1</v>
       </c>
       <c r="K40" s="7">
@@ -4864,7 +4897,7 @@
       </c>
       <c r="P40" s="14">
         <f t="shared" si="3"/>
-        <v>0.67</v>
+        <v>3.35</v>
       </c>
       <c r="Q40" s="14">
         <v>0.45290000000000002</v>
@@ -4888,15 +4921,15 @@
       <c r="A41" s="28">
         <v>39</v>
       </c>
-      <c r="B41" s="42"/>
-      <c r="C41" s="58" t="s">
-        <v>246</v>
+      <c r="B41" s="137"/>
+      <c r="C41" s="49" t="s">
+        <v>245</v>
       </c>
       <c r="D41" s="24" t="s">
         <v>60</v>
       </c>
       <c r="E41" s="21" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F41" s="24" t="s">
         <v>189</v>
@@ -4910,7 +4943,7 @@
       <c r="I41" s="24" t="s">
         <v>222</v>
       </c>
-      <c r="J41" s="48">
+      <c r="J41" s="39">
         <v>1</v>
       </c>
       <c r="K41" s="7">
@@ -4933,7 +4966,7 @@
       </c>
       <c r="P41" s="14">
         <f t="shared" si="3"/>
-        <v>0.41</v>
+        <v>2.0499999999999998</v>
       </c>
       <c r="Q41" s="14">
         <v>0.17380000000000001</v>
@@ -4957,21 +4990,21 @@
       <c r="A42" s="28">
         <v>40</v>
       </c>
-      <c r="B42" s="42"/>
-      <c r="C42" s="58" t="s">
+      <c r="B42" s="137"/>
+      <c r="C42" s="49" t="s">
         <v>71</v>
       </c>
       <c r="D42" s="24" t="s">
         <v>7</v>
       </c>
       <c r="E42" s="24" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="F42" s="24" t="s">
         <v>63</v>
       </c>
       <c r="G42" s="24" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="H42" s="24" t="s">
         <v>222</v>
@@ -4979,7 +5012,7 @@
       <c r="I42" s="24" t="s">
         <v>222</v>
       </c>
-      <c r="J42" s="48">
+      <c r="J42" s="39">
         <v>1</v>
       </c>
       <c r="K42" s="7">
@@ -4995,14 +5028,14 @@
         <v>1000</v>
       </c>
       <c r="N42" s="27" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="O42" s="14">
         <v>0.51</v>
       </c>
       <c r="P42" s="14">
         <f t="shared" si="3"/>
-        <v>0.51</v>
+        <v>2.5499999999999998</v>
       </c>
       <c r="Q42" s="14">
         <v>0.30599999999999999</v>
@@ -5026,69 +5059,69 @@
       <c r="A43" s="28">
         <v>41</v>
       </c>
-      <c r="B43" s="42"/>
-      <c r="C43" s="135" t="s">
+      <c r="B43" s="137"/>
+      <c r="C43" s="122" t="s">
+        <v>248</v>
+      </c>
+      <c r="D43" s="68" t="s">
+        <v>36</v>
+      </c>
+      <c r="E43" s="70" t="s">
         <v>249</v>
       </c>
-      <c r="D43" s="79" t="s">
-        <v>36</v>
-      </c>
-      <c r="E43" s="81" t="s">
-        <v>250</v>
-      </c>
-      <c r="F43" s="79" t="s">
+      <c r="F43" s="68" t="s">
         <v>190</v>
       </c>
-      <c r="G43" s="79" t="s">
-        <v>248</v>
-      </c>
-      <c r="H43" s="79" t="s">
-        <v>222</v>
-      </c>
-      <c r="I43" s="79" t="s">
-        <v>222</v>
-      </c>
-      <c r="J43" s="82">
+      <c r="G43" s="68" t="s">
+        <v>247</v>
+      </c>
+      <c r="H43" s="68" t="s">
+        <v>222</v>
+      </c>
+      <c r="I43" s="68" t="s">
+        <v>222</v>
+      </c>
+      <c r="J43" s="71">
         <v>1</v>
       </c>
-      <c r="K43" s="49">
+      <c r="K43" s="40">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L43" s="49">
+      <c r="L43" s="40">
         <f t="shared" si="1"/>
         <v>100</v>
       </c>
-      <c r="M43" s="49">
+      <c r="M43" s="40">
         <f t="shared" si="2"/>
         <v>1000</v>
       </c>
-      <c r="N43" s="83" t="s">
-        <v>257</v>
-      </c>
-      <c r="O43" s="84">
+      <c r="N43" s="72" t="s">
+        <v>256</v>
+      </c>
+      <c r="O43" s="73">
         <v>2.6688999999999998</v>
       </c>
-      <c r="P43" s="84">
+      <c r="P43" s="14">
         <f t="shared" si="3"/>
+        <v>13.3445</v>
+      </c>
+      <c r="Q43" s="73">
         <v>2.6688999999999998</v>
       </c>
-      <c r="Q43" s="84">
-        <v>2.6688999999999998</v>
-      </c>
-      <c r="R43" s="84">
+      <c r="R43" s="73">
         <f t="shared" si="4"/>
         <v>266.89</v>
       </c>
-      <c r="S43" s="84">
+      <c r="S43" s="73">
         <v>0.97919999999999996</v>
       </c>
-      <c r="T43" s="84">
+      <c r="T43" s="73">
         <f t="shared" si="5"/>
         <v>979.19999999999993</v>
       </c>
-      <c r="U43" s="94" t="s">
-        <v>281</v>
+      <c r="U43" s="82" t="s">
+        <v>280</v>
       </c>
       <c r="V43" s="3"/>
       <c r="W43" s="3"/>
@@ -5097,69 +5130,69 @@
       <c r="A44" s="28">
         <v>42</v>
       </c>
-      <c r="B44" s="42"/>
-      <c r="C44" s="135" t="s">
-        <v>253</v>
-      </c>
-      <c r="D44" s="79" t="s">
+      <c r="B44" s="137"/>
+      <c r="C44" s="122" t="s">
+        <v>252</v>
+      </c>
+      <c r="D44" s="68" t="s">
         <v>37</v>
       </c>
-      <c r="E44" s="81" t="s">
-        <v>252</v>
-      </c>
-      <c r="F44" s="79" t="s">
+      <c r="E44" s="70" t="s">
+        <v>251</v>
+      </c>
+      <c r="F44" s="68" t="s">
         <v>191</v>
       </c>
-      <c r="G44" s="79" t="s">
-        <v>248</v>
-      </c>
-      <c r="H44" s="79" t="s">
-        <v>222</v>
-      </c>
-      <c r="I44" s="79" t="s">
-        <v>222</v>
-      </c>
-      <c r="J44" s="82">
+      <c r="G44" s="68" t="s">
+        <v>247</v>
+      </c>
+      <c r="H44" s="68" t="s">
+        <v>222</v>
+      </c>
+      <c r="I44" s="68" t="s">
+        <v>222</v>
+      </c>
+      <c r="J44" s="71">
         <v>1</v>
       </c>
-      <c r="K44" s="49">
+      <c r="K44" s="40">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L44" s="49">
+      <c r="L44" s="40">
         <f t="shared" si="1"/>
         <v>100</v>
       </c>
-      <c r="M44" s="49">
+      <c r="M44" s="40">
         <f t="shared" si="2"/>
         <v>1000</v>
       </c>
-      <c r="N44" s="83" t="s">
-        <v>257</v>
-      </c>
-      <c r="O44" s="84">
+      <c r="N44" s="72" t="s">
+        <v>256</v>
+      </c>
+      <c r="O44" s="73">
         <v>2.0756000000000001</v>
       </c>
-      <c r="P44" s="84">
+      <c r="P44" s="14">
         <f t="shared" si="3"/>
-        <v>2.0756000000000001</v>
-      </c>
-      <c r="Q44" s="84">
+        <v>10.378</v>
+      </c>
+      <c r="Q44" s="73">
         <v>1.3399000000000001</v>
       </c>
-      <c r="R44" s="84">
+      <c r="R44" s="73">
         <f t="shared" si="4"/>
         <v>133.99</v>
       </c>
-      <c r="S44" s="84">
+      <c r="S44" s="73">
         <v>1.2749999999999999</v>
       </c>
-      <c r="T44" s="84">
+      <c r="T44" s="73">
         <f t="shared" si="5"/>
         <v>1275</v>
       </c>
-      <c r="U44" s="94" t="s">
-        <v>281</v>
+      <c r="U44" s="82" t="s">
+        <v>280</v>
       </c>
       <c r="V44" s="3"/>
       <c r="W44" s="3"/>
@@ -5168,69 +5201,69 @@
       <c r="A45" s="28">
         <v>43</v>
       </c>
-      <c r="B45" s="43"/>
-      <c r="C45" s="108" t="s">
+      <c r="B45" s="138"/>
+      <c r="C45" s="95" t="s">
         <v>192</v>
       </c>
-      <c r="D45" s="109" t="s">
+      <c r="D45" s="96" t="s">
         <v>193</v>
       </c>
-      <c r="E45" s="110" t="s">
-        <v>251</v>
-      </c>
-      <c r="F45" s="109" t="s">
+      <c r="E45" s="97" t="s">
+        <v>250</v>
+      </c>
+      <c r="F45" s="96" t="s">
         <v>194</v>
       </c>
-      <c r="G45" s="109" t="s">
-        <v>271</v>
-      </c>
-      <c r="H45" s="109" t="s">
-        <v>222</v>
-      </c>
-      <c r="I45" s="109" t="s">
-        <v>222</v>
-      </c>
-      <c r="J45" s="112">
+      <c r="G45" s="96" t="s">
+        <v>270</v>
+      </c>
+      <c r="H45" s="96" t="s">
+        <v>222</v>
+      </c>
+      <c r="I45" s="96" t="s">
+        <v>222</v>
+      </c>
+      <c r="J45" s="99">
         <v>1</v>
       </c>
-      <c r="K45" s="113">
+      <c r="K45" s="100">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L45" s="113">
+      <c r="L45" s="100">
         <f t="shared" si="1"/>
         <v>100</v>
       </c>
-      <c r="M45" s="113">
+      <c r="M45" s="100">
         <f t="shared" si="2"/>
         <v>1000</v>
       </c>
-      <c r="N45" s="114" t="s">
-        <v>257</v>
-      </c>
-      <c r="O45" s="115">
+      <c r="N45" s="101" t="s">
+        <v>256</v>
+      </c>
+      <c r="O45" s="102">
         <v>2.0129999999999999</v>
       </c>
-      <c r="P45" s="115">
+      <c r="P45" s="15">
         <f t="shared" si="3"/>
-        <v>2.0129999999999999</v>
-      </c>
-      <c r="Q45" s="115">
+        <v>10.065</v>
+      </c>
+      <c r="Q45" s="102">
         <v>1.4630000000000001</v>
       </c>
-      <c r="R45" s="115">
+      <c r="R45" s="102">
         <f t="shared" si="4"/>
         <v>146.30000000000001</v>
       </c>
-      <c r="S45" s="115">
+      <c r="S45" s="102">
         <v>1.4139999999999999</v>
       </c>
-      <c r="T45" s="115">
+      <c r="T45" s="102">
         <f t="shared" si="5"/>
         <v>1414</v>
       </c>
-      <c r="U45" s="133" t="s">
-        <v>281</v>
+      <c r="U45" s="120" t="s">
+        <v>280</v>
       </c>
       <c r="V45" s="3"/>
       <c r="W45" s="3"/>
@@ -5239,70 +5272,70 @@
       <c r="A46" s="28">
         <v>44</v>
       </c>
-      <c r="B46" s="40" t="s">
-        <v>254</v>
-      </c>
-      <c r="C46" s="120" t="s">
+      <c r="B46" s="132" t="s">
+        <v>253</v>
+      </c>
+      <c r="C46" s="107" t="s">
         <v>195</v>
       </c>
-      <c r="D46" s="121" t="s">
+      <c r="D46" s="108" t="s">
         <v>59</v>
       </c>
-      <c r="E46" s="121" t="s">
+      <c r="E46" s="108" t="s">
         <v>108</v>
       </c>
-      <c r="F46" s="121" t="s">
+      <c r="F46" s="108" t="s">
         <v>196</v>
       </c>
-      <c r="G46" s="121" t="s">
+      <c r="G46" s="108" t="s">
+        <v>271</v>
+      </c>
+      <c r="H46" s="109" t="s">
         <v>272</v>
       </c>
-      <c r="H46" s="122" t="s">
+      <c r="I46" s="109" t="s">
         <v>273</v>
       </c>
-      <c r="I46" s="122" t="s">
-        <v>274</v>
-      </c>
-      <c r="J46" s="123">
+      <c r="J46" s="110">
         <v>1</v>
       </c>
-      <c r="K46" s="124">
+      <c r="K46" s="111">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L46" s="124">
+      <c r="L46" s="111">
         <f t="shared" si="1"/>
         <v>100</v>
       </c>
-      <c r="M46" s="124">
+      <c r="M46" s="111">
         <f t="shared" si="2"/>
         <v>1000</v>
       </c>
-      <c r="N46" s="125" t="s">
-        <v>257</v>
-      </c>
-      <c r="O46" s="126">
+      <c r="N46" s="112" t="s">
+        <v>256</v>
+      </c>
+      <c r="O46" s="113">
         <v>0.28570000000000001</v>
       </c>
-      <c r="P46" s="126">
+      <c r="P46" s="150">
         <f t="shared" si="3"/>
-        <v>0.28570000000000001</v>
-      </c>
-      <c r="Q46" s="126">
+        <v>1.4285000000000001</v>
+      </c>
+      <c r="Q46" s="113">
         <v>0.1459</v>
       </c>
-      <c r="R46" s="126">
+      <c r="R46" s="113">
         <f t="shared" si="4"/>
         <v>14.59</v>
       </c>
-      <c r="S46" s="126">
+      <c r="S46" s="113">
         <v>0.13980000000000001</v>
       </c>
-      <c r="T46" s="126">
+      <c r="T46" s="113">
         <f t="shared" si="5"/>
         <v>139.80000000000001</v>
       </c>
-      <c r="U46" s="127"/>
+      <c r="U46" s="114"/>
       <c r="V46" s="3"/>
       <c r="W46" s="3"/>
     </row>
@@ -5310,71 +5343,71 @@
       <c r="A47" s="28">
         <v>45</v>
       </c>
-      <c r="B47" s="41" t="s">
+      <c r="B47" s="136" t="s">
         <v>76</v>
       </c>
-      <c r="C47" s="96" t="s">
+      <c r="C47" s="83" t="s">
         <v>197</v>
       </c>
-      <c r="D47" s="86" t="s">
+      <c r="D47" s="75" t="s">
         <v>5</v>
       </c>
-      <c r="E47" s="86" t="s">
+      <c r="E47" s="75" t="s">
         <v>108</v>
       </c>
-      <c r="F47" s="86" t="s">
+      <c r="F47" s="75" t="s">
         <v>198</v>
       </c>
-      <c r="G47" s="87" t="s">
-        <v>269</v>
-      </c>
-      <c r="H47" s="87" t="s">
+      <c r="G47" s="76" t="s">
+        <v>268</v>
+      </c>
+      <c r="H47" s="76" t="s">
+        <v>281</v>
+      </c>
+      <c r="I47" s="76" t="s">
         <v>282</v>
       </c>
-      <c r="I47" s="87" t="s">
-        <v>283</v>
-      </c>
-      <c r="J47" s="97">
+      <c r="J47" s="84">
         <v>1</v>
       </c>
-      <c r="K47" s="89">
+      <c r="K47" s="78">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L47" s="89">
+      <c r="L47" s="78">
         <f t="shared" si="1"/>
         <v>100</v>
       </c>
-      <c r="M47" s="89">
+      <c r="M47" s="78">
         <f t="shared" si="2"/>
         <v>1000</v>
       </c>
-      <c r="N47" s="136" t="s">
-        <v>257</v>
-      </c>
-      <c r="O47" s="137">
+      <c r="N47" s="123" t="s">
+        <v>256</v>
+      </c>
+      <c r="O47" s="124">
         <v>0.74480000000000002</v>
       </c>
-      <c r="P47" s="91">
+      <c r="P47" s="13">
         <f t="shared" si="3"/>
-        <v>0.74480000000000002</v>
-      </c>
-      <c r="Q47" s="137">
+        <v>3.7240000000000002</v>
+      </c>
+      <c r="Q47" s="124">
         <v>0.41560000000000002</v>
       </c>
-      <c r="R47" s="91">
+      <c r="R47" s="80">
         <f t="shared" si="4"/>
         <v>41.56</v>
       </c>
-      <c r="S47" s="91">
+      <c r="S47" s="80">
         <v>0.39279999999999998</v>
       </c>
-      <c r="T47" s="91">
+      <c r="T47" s="80">
         <f t="shared" si="5"/>
         <v>392.79999999999995</v>
       </c>
-      <c r="U47" s="132" t="s">
-        <v>281</v>
+      <c r="U47" s="119" t="s">
+        <v>280</v>
       </c>
       <c r="V47" s="3"/>
       <c r="W47" s="3"/>
@@ -5383,68 +5416,68 @@
       <c r="A48" s="28">
         <v>46</v>
       </c>
-      <c r="B48" s="42"/>
-      <c r="C48" s="78" t="s">
+      <c r="B48" s="137"/>
+      <c r="C48" s="67" t="s">
         <v>199</v>
       </c>
-      <c r="D48" s="79" t="s">
+      <c r="D48" s="68" t="s">
         <v>200</v>
       </c>
-      <c r="E48" s="79" t="s">
+      <c r="E48" s="68" t="s">
         <v>108</v>
       </c>
-      <c r="F48" s="79" t="s">
+      <c r="F48" s="68" t="s">
         <v>201</v>
       </c>
-      <c r="G48" s="80" t="s">
-        <v>275</v>
-      </c>
-      <c r="H48" s="79" t="s">
-        <v>222</v>
-      </c>
-      <c r="I48" s="79" t="s">
-        <v>222</v>
-      </c>
-      <c r="J48" s="128">
+      <c r="G48" s="69" t="s">
+        <v>274</v>
+      </c>
+      <c r="H48" s="68" t="s">
+        <v>222</v>
+      </c>
+      <c r="I48" s="68" t="s">
+        <v>222</v>
+      </c>
+      <c r="J48" s="115">
         <v>2</v>
       </c>
-      <c r="K48" s="49">
+      <c r="K48" s="40">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="L48" s="49">
+      <c r="L48" s="40">
         <f t="shared" si="1"/>
         <v>200</v>
       </c>
-      <c r="M48" s="49">
+      <c r="M48" s="40">
         <f t="shared" si="2"/>
         <v>2000</v>
       </c>
-      <c r="N48" s="129" t="s">
-        <v>257</v>
-      </c>
-      <c r="O48" s="84">
+      <c r="N48" s="116" t="s">
+        <v>256</v>
+      </c>
+      <c r="O48" s="73">
         <v>4.4699999999999997E-2</v>
       </c>
-      <c r="P48" s="84">
+      <c r="P48" s="14">
         <f t="shared" si="3"/>
-        <v>8.9399999999999993E-2</v>
-      </c>
-      <c r="Q48" s="84">
+        <v>0.44699999999999995</v>
+      </c>
+      <c r="Q48" s="73">
         <v>3.39E-2</v>
       </c>
-      <c r="R48" s="84">
+      <c r="R48" s="73">
         <f t="shared" si="4"/>
         <v>6.78</v>
       </c>
-      <c r="S48" s="84">
+      <c r="S48" s="73">
         <v>2.4E-2</v>
       </c>
-      <c r="T48" s="84">
+      <c r="T48" s="73">
         <f t="shared" si="5"/>
         <v>48</v>
       </c>
-      <c r="U48" s="37"/>
+      <c r="U48" s="36"/>
       <c r="V48" s="3"/>
       <c r="W48" s="3"/>
     </row>
@@ -5452,68 +5485,68 @@
       <c r="A49" s="28">
         <v>47</v>
       </c>
-      <c r="B49" s="42"/>
-      <c r="C49" s="78" t="s">
+      <c r="B49" s="137"/>
+      <c r="C49" s="67" t="s">
         <v>202</v>
       </c>
-      <c r="D49" s="79" t="s">
+      <c r="D49" s="68" t="s">
         <v>203</v>
       </c>
-      <c r="E49" s="79" t="s">
+      <c r="E49" s="68" t="s">
         <v>108</v>
       </c>
-      <c r="F49" s="79" t="s">
+      <c r="F49" s="68" t="s">
         <v>204</v>
       </c>
-      <c r="G49" s="80" t="s">
-        <v>269</v>
-      </c>
-      <c r="H49" s="79" t="s">
-        <v>222</v>
-      </c>
-      <c r="I49" s="79" t="s">
-        <v>222</v>
-      </c>
-      <c r="J49" s="130">
+      <c r="G49" s="69" t="s">
+        <v>268</v>
+      </c>
+      <c r="H49" s="68" t="s">
+        <v>222</v>
+      </c>
+      <c r="I49" s="68" t="s">
+        <v>222</v>
+      </c>
+      <c r="J49" s="117">
         <v>1</v>
       </c>
-      <c r="K49" s="49">
+      <c r="K49" s="40">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L49" s="49">
+      <c r="L49" s="40">
         <f t="shared" si="1"/>
         <v>100</v>
       </c>
-      <c r="M49" s="49">
+      <c r="M49" s="40">
         <f t="shared" si="2"/>
         <v>1000</v>
       </c>
-      <c r="N49" s="129" t="s">
-        <v>257</v>
-      </c>
-      <c r="O49" s="84">
+      <c r="N49" s="116" t="s">
+        <v>256</v>
+      </c>
+      <c r="O49" s="73">
         <v>0.11650000000000001</v>
       </c>
-      <c r="P49" s="84">
+      <c r="P49" s="14">
         <f t="shared" si="3"/>
-        <v>0.11650000000000001</v>
-      </c>
-      <c r="Q49" s="84">
+        <v>0.58250000000000002</v>
+      </c>
+      <c r="Q49" s="73">
         <v>8.4099999999999994E-2</v>
       </c>
-      <c r="R49" s="84">
+      <c r="R49" s="73">
         <f t="shared" si="4"/>
         <v>8.41</v>
       </c>
-      <c r="S49" s="84">
+      <c r="S49" s="73">
         <v>3.61E-2</v>
       </c>
-      <c r="T49" s="84">
+      <c r="T49" s="73">
         <f t="shared" si="5"/>
         <v>36.1</v>
       </c>
-      <c r="U49" s="131"/>
+      <c r="U49" s="118"/>
       <c r="V49" s="3"/>
       <c r="W49" s="3"/>
     </row>
@@ -5521,8 +5554,8 @@
       <c r="A50" s="28">
         <v>48</v>
       </c>
-      <c r="B50" s="42"/>
-      <c r="C50" s="56" t="s">
+      <c r="B50" s="137"/>
+      <c r="C50" s="47" t="s">
         <v>205</v>
       </c>
       <c r="D50" s="24" t="s">
@@ -5543,7 +5576,7 @@
       <c r="I50" s="24" t="s">
         <v>222</v>
       </c>
-      <c r="J50" s="34">
+      <c r="J50" s="33">
         <v>1</v>
       </c>
       <c r="K50" s="7">
@@ -5558,7 +5591,7 @@
         <f t="shared" si="2"/>
         <v>1000</v>
       </c>
-      <c r="N50" s="31" t="s">
+      <c r="N50" s="30" t="s">
         <v>17</v>
       </c>
       <c r="O50" s="14">
@@ -5566,7 +5599,7 @@
       </c>
       <c r="P50" s="14">
         <f t="shared" si="3"/>
-        <v>0.34</v>
+        <v>1.7000000000000002</v>
       </c>
       <c r="Q50" s="14">
         <v>0.182</v>
@@ -5587,32 +5620,32 @@
       <c r="W50" s="3"/>
     </row>
     <row r="51" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="29">
+      <c r="A51" s="28">
         <v>49</v>
       </c>
-      <c r="B51" s="43"/>
-      <c r="C51" s="62" t="s">
+      <c r="B51" s="138"/>
+      <c r="C51" s="52" t="s">
         <v>209</v>
       </c>
-      <c r="D51" s="63" t="s">
+      <c r="D51" s="53" t="s">
         <v>210</v>
       </c>
-      <c r="E51" s="63" t="s">
+      <c r="E51" s="53" t="s">
         <v>211</v>
       </c>
-      <c r="F51" s="63" t="s">
+      <c r="F51" s="53" t="s">
         <v>212</v>
       </c>
       <c r="G51" s="9" t="s">
-        <v>255</v>
-      </c>
-      <c r="H51" s="63" t="s">
-        <v>222</v>
-      </c>
-      <c r="I51" s="63" t="s">
-        <v>222</v>
-      </c>
-      <c r="J51" s="39">
+        <v>254</v>
+      </c>
+      <c r="H51" s="53" t="s">
+        <v>222</v>
+      </c>
+      <c r="I51" s="53" t="s">
+        <v>222</v>
+      </c>
+      <c r="J51" s="38">
         <v>1</v>
       </c>
       <c r="K51" s="10">
@@ -5627,15 +5660,15 @@
         <f t="shared" si="2"/>
         <v>1000</v>
       </c>
-      <c r="N51" s="38" t="s">
-        <v>256</v>
+      <c r="N51" s="37" t="s">
+        <v>255</v>
       </c>
       <c r="O51" s="15">
         <v>0.23719999999999999</v>
       </c>
-      <c r="P51" s="15">
+      <c r="P51" s="143">
         <f t="shared" si="3"/>
-        <v>0.23719999999999999</v>
+        <v>1.1859999999999999</v>
       </c>
       <c r="Q51" s="15">
         <v>0.2021</v>
@@ -5656,45 +5689,49 @@
       <c r="W51" s="3"/>
     </row>
     <row r="52" spans="1:23" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="K52" s="44" t="s">
+      <c r="K52" s="139" t="s">
         <v>18</v>
       </c>
-      <c r="L52" s="44"/>
-      <c r="M52" s="44"/>
-      <c r="N52" s="44"/>
-      <c r="P52" s="59">
+      <c r="L52" s="139"/>
+      <c r="M52" s="139"/>
+      <c r="N52" s="139"/>
+      <c r="P52" s="29">
         <f>SUM(P3:P51)</f>
-        <v>29.316200000000002</v>
+        <v>134.48999999999998</v>
       </c>
       <c r="Q52" s="16"/>
-      <c r="R52" s="30">
+      <c r="R52" s="29">
         <f>SUM(R3:R51)</f>
-        <v>1803.4679999999998</v>
+        <v>1769.6680000000001</v>
       </c>
       <c r="S52" s="17"/>
-      <c r="T52" s="30">
+      <c r="T52" s="29">
         <f>SUM(T3:T51)</f>
-        <v>13220.659999999998</v>
+        <v>13049.46</v>
       </c>
       <c r="V52" s="3"/>
       <c r="W52" s="3"/>
     </row>
     <row r="53" spans="1:23" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K53" s="77" t="s">
+      <c r="K53" s="140" t="s">
         <v>19</v>
       </c>
-      <c r="L53" s="77"/>
-      <c r="M53" s="77"/>
-      <c r="N53" s="77"/>
+      <c r="L53" s="140"/>
+      <c r="M53" s="140"/>
+      <c r="N53" s="140"/>
+      <c r="P53" s="141">
+        <f>P52/5</f>
+        <v>26.897999999999996</v>
+      </c>
       <c r="Q53" s="17"/>
       <c r="R53" s="18">
         <f>R52/100</f>
-        <v>18.034679999999998</v>
+        <v>17.696680000000001</v>
       </c>
       <c r="S53" s="18"/>
       <c r="T53" s="18">
         <f>T52/1000</f>
-        <v>13.220659999999999</v>
+        <v>13.04946</v>
       </c>
       <c r="V53" s="3"/>
       <c r="W53" s="3"/>
@@ -5828,7 +5865,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P3:P51">
+  <conditionalFormatting sqref="P3:P51 P53">
     <cfRule type="dataBar" priority="91">
       <dataBar>
         <cfvo type="min"/>
@@ -5901,51 +5938,51 @@
     <hyperlink ref="N6" r:id="rId2"/>
     <hyperlink ref="N7" r:id="rId3"/>
     <hyperlink ref="N8" r:id="rId4"/>
-    <hyperlink ref="N9" r:id="rId5"/>
-    <hyperlink ref="N10" r:id="rId6"/>
-    <hyperlink ref="N13" r:id="rId7"/>
-    <hyperlink ref="N15" r:id="rId8"/>
-    <hyperlink ref="N16" r:id="rId9"/>
-    <hyperlink ref="N19" r:id="rId10"/>
-    <hyperlink ref="N22" r:id="rId11"/>
-    <hyperlink ref="N23" r:id="rId12"/>
-    <hyperlink ref="N24" r:id="rId13"/>
-    <hyperlink ref="N26" r:id="rId14"/>
-    <hyperlink ref="N28" r:id="rId15"/>
-    <hyperlink ref="N29" r:id="rId16"/>
-    <hyperlink ref="N30" r:id="rId17"/>
-    <hyperlink ref="N31" r:id="rId18"/>
-    <hyperlink ref="N32" r:id="rId19"/>
-    <hyperlink ref="N33" r:id="rId20"/>
-    <hyperlink ref="N34" r:id="rId21"/>
-    <hyperlink ref="N36" r:id="rId22"/>
-    <hyperlink ref="N39" r:id="rId23"/>
-    <hyperlink ref="N40" r:id="rId24"/>
-    <hyperlink ref="N41" r:id="rId25"/>
-    <hyperlink ref="N42" r:id="rId26"/>
-    <hyperlink ref="N50" r:id="rId27"/>
-    <hyperlink ref="N51" r:id="rId28"/>
-    <hyperlink ref="N5" r:id="rId29"/>
-    <hyperlink ref="N11" r:id="rId30"/>
-    <hyperlink ref="N12" r:id="rId31"/>
-    <hyperlink ref="N14" r:id="rId32"/>
-    <hyperlink ref="N17" r:id="rId33"/>
-    <hyperlink ref="N20" r:id="rId34"/>
-    <hyperlink ref="N21" r:id="rId35"/>
-    <hyperlink ref="N25" r:id="rId36"/>
-    <hyperlink ref="N27" r:id="rId37"/>
-    <hyperlink ref="N35" r:id="rId38"/>
-    <hyperlink ref="N38" r:id="rId39"/>
-    <hyperlink ref="N46" r:id="rId40"/>
-    <hyperlink ref="N48" r:id="rId41"/>
-    <hyperlink ref="N49" r:id="rId42"/>
-    <hyperlink ref="N4" r:id="rId43"/>
-    <hyperlink ref="N18" r:id="rId44"/>
-    <hyperlink ref="N37" r:id="rId45"/>
-    <hyperlink ref="N43" r:id="rId46"/>
-    <hyperlink ref="N44" r:id="rId47"/>
-    <hyperlink ref="N45" r:id="rId48"/>
-    <hyperlink ref="N47" r:id="rId49"/>
+    <hyperlink ref="N10" r:id="rId5"/>
+    <hyperlink ref="N13" r:id="rId6"/>
+    <hyperlink ref="N15" r:id="rId7"/>
+    <hyperlink ref="N16" r:id="rId8"/>
+    <hyperlink ref="N19" r:id="rId9"/>
+    <hyperlink ref="N22" r:id="rId10"/>
+    <hyperlink ref="N23" r:id="rId11"/>
+    <hyperlink ref="N24" r:id="rId12"/>
+    <hyperlink ref="N26" r:id="rId13"/>
+    <hyperlink ref="N28" r:id="rId14"/>
+    <hyperlink ref="N29" r:id="rId15"/>
+    <hyperlink ref="N30" r:id="rId16"/>
+    <hyperlink ref="N31" r:id="rId17"/>
+    <hyperlink ref="N32" r:id="rId18"/>
+    <hyperlink ref="N33" r:id="rId19"/>
+    <hyperlink ref="N34" r:id="rId20"/>
+    <hyperlink ref="N36" r:id="rId21"/>
+    <hyperlink ref="N39" r:id="rId22"/>
+    <hyperlink ref="N40" r:id="rId23"/>
+    <hyperlink ref="N41" r:id="rId24"/>
+    <hyperlink ref="N42" r:id="rId25"/>
+    <hyperlink ref="N50" r:id="rId26"/>
+    <hyperlink ref="N51" r:id="rId27"/>
+    <hyperlink ref="N5" r:id="rId28"/>
+    <hyperlink ref="N11" r:id="rId29"/>
+    <hyperlink ref="N12" r:id="rId30"/>
+    <hyperlink ref="N14" r:id="rId31"/>
+    <hyperlink ref="N17" r:id="rId32"/>
+    <hyperlink ref="N20" r:id="rId33"/>
+    <hyperlink ref="N21" r:id="rId34"/>
+    <hyperlink ref="N25" r:id="rId35"/>
+    <hyperlink ref="N27" r:id="rId36"/>
+    <hyperlink ref="N35" r:id="rId37"/>
+    <hyperlink ref="N38" r:id="rId38"/>
+    <hyperlink ref="N46" r:id="rId39"/>
+    <hyperlink ref="N48" r:id="rId40"/>
+    <hyperlink ref="N49" r:id="rId41"/>
+    <hyperlink ref="N4" r:id="rId42"/>
+    <hyperlink ref="N18" r:id="rId43"/>
+    <hyperlink ref="N37" r:id="rId44"/>
+    <hyperlink ref="N43" r:id="rId45"/>
+    <hyperlink ref="N44" r:id="rId46"/>
+    <hyperlink ref="N45" r:id="rId47"/>
+    <hyperlink ref="N47" r:id="rId48"/>
+    <hyperlink ref="N9" r:id="rId49"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId50"/>
@@ -6028,7 +6065,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>P3:P51</xm:sqref>
+          <xm:sqref>P3:P51 P53</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{2F6B6F4F-BC31-4B63-B3A8-F7820745DC3B}">

</xml_diff>